<commit_message>
run data: the mean of each measure per arm
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finished_data/grag-data.xlsx
+++ b/finished_data/grag-data.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'results'!$A$1:$AC$301</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'arm construction'!$A$1:$D$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -28932,13 +28932,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -29123,6 +29123,388 @@
       </c>
       <c r="D14" t="n">
         <v>4198.130214499775</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>mean of</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>lucene</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>artefact</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>faithfulness</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.89812279853706</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.8623698038810772</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.9049227200847346</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>answer_correctness</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.174588395260194</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.2170203676255874</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.2729603400642577</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>context_recall_id</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.0913227669812124</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.2356876416725427</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.6470207819231475</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>context_precision_id</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.05496487066333602</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.0625631727534575</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.193456257106725</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>context_recall_llm</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.2533333333333333</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.4464047619047619</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.6059848484848485</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>context_recall_nonllm</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.07347356884306215</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.1741445532778351</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.0528971948824701</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>context_precision_nonllm</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0.1757800623422777</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.1945623840642109</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.1947211814750251</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>semantic_similarity</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.327001708564771</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.3295387992718101</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.3754341377738559</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>string_similarity</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.1307197821004649</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.1133058591546737</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.1177289717073062</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>bleu</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.02490116032934318</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.0185879762537921</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.02762799978000487</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>rouge</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.09673166490384025</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.1027315257536634</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.1274620748666058</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>chrf</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0.2099397290459472</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.2183964674831196</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.2632451489979341</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>exact_match</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>string_presence</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>search_seconds</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.0304097359883599</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.06788752002175898</v>
+      </c>
+      <c r="D31" t="n">
+        <v>2.209680197946727</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>interpreter_seconds</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>13.55906191201415</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>query_embedding_seconds</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>0.4786859189951793</v>
+      </c>
+      <c r="D33" t="n">
+        <v>2.866435058019124</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>answer_seconds</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>6.749374916995875</v>
+      </c>
+      <c r="C34" t="n">
+        <v>8.107556761973537</v>
+      </c>
+      <c r="D34" t="n">
+        <v>7.416482453998178</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>total_seconds</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>6.787730676007922</v>
+      </c>
+      <c r="C35" t="n">
+        <v>8.667278056973592</v>
+      </c>
+      <c r="D35" t="n">
+        <v>26.05431466102134</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>interpreter_tokens_in</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>3257.76</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>interpreter_tokens_out</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1009.25</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>query_embedding_tokens</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>22.08</v>
+      </c>
+      <c r="D38" t="n">
+        <v>108.69</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>answer_tokens_in</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>26281.19</v>
+      </c>
+      <c r="C39" t="n">
+        <v>30165.13</v>
+      </c>
+      <c r="D39" t="n">
+        <v>32440.12</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>answer_tokens_out</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>317.86</v>
+      </c>
+      <c r="C40" t="n">
+        <v>427.55</v>
+      </c>
+      <c r="D40" t="n">
+        <v>373.96</v>
       </c>
     </row>
   </sheetData>
@@ -29384,7 +29766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -30222,17 +30604,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>arm construction</t>
+          <t>run data</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>mean of</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Index type.</t>
+          <t>Mean over the arm's 100 questions of the field of results named in the row.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -30245,12 +30627,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>index</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Unit stored in the index.</t>
+          <t>Index type.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -30263,19 +30645,15 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>units in the index</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Units in the index.</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
+          <t>Unit stored in the index.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -30285,17 +30663,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>build time, seconds</t>
+          <t>units in the index</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Time to build the index. Artefact: sum of the times of the build steps.</t>
+          <t>Units in the index.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>seconds</t>
+          <t>count</t>
         </is>
       </c>
     </row>
@@ -30307,17 +30685,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
+          <t>build time, seconds</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Texts embedded for the index.</t>
+          <t>Time to build the index. Artefact: sum of the times of the build steps.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
@@ -30329,17 +30707,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, tokens</t>
+          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Tokens embedded for the index.</t>
+          <t>Texts embedded for the index.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>count</t>
         </is>
       </c>
     </row>
@@ -30351,17 +30729,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, seconds</t>
+          <t>llama-nemotron-embed-1b-v2, tokens</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Embedding time for the index.</t>
+          <t>Tokens embedded for the index.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>seconds</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
@@ -30373,17 +30751,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, calls</t>
+          <t>llama-nemotron-embed-1b-v2, seconds</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Calls to claude-haiku-4-5 for the index.</t>
+          <t>Embedding time for the index.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
@@ -30395,17 +30773,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, tokens in</t>
+          <t>claude-haiku-4-5, calls</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Input tokens of those calls.</t>
+          <t>Calls to claude-haiku-4-5 for the index.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>count</t>
         </is>
       </c>
     </row>
@@ -30417,12 +30795,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, tokens out</t>
+          <t>claude-haiku-4-5, tokens in</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Output tokens of those calls.</t>
+          <t>Input tokens of those calls.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -30439,17 +30817,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, seconds</t>
+          <t>claude-haiku-4-5, tokens out</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Time of those calls: the time of the pass that made them, multiplied by their share of the pass's call time.</t>
+          <t>Output tokens of those calls.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>seconds</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
@@ -30461,17 +30839,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>claude-opus-5, calls</t>
+          <t>claude-haiku-4-5, seconds</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Calls to claude-opus-5 for the index.</t>
+          <t>Time of those calls: the time of the pass that made them, multiplied by their share of the pass's call time.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
@@ -30483,17 +30861,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>claude-opus-5, tokens in</t>
+          <t>claude-opus-5, calls</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Input tokens of those calls.</t>
+          <t>Calls to claude-opus-5 for the index.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>count</t>
         </is>
       </c>
     </row>
@@ -30505,12 +30883,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>claude-opus-5, tokens out</t>
+          <t>claude-opus-5, tokens in</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Output tokens of those calls.</t>
+          <t>Input tokens of those calls.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -30527,17 +30905,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>claude-opus-5, seconds</t>
+          <t>claude-opus-5, tokens out</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Time of those calls.</t>
+          <t>Output tokens of those calls.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>seconds</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
@@ -30549,22 +30927,44 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>claude-opus-5, seconds</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Time of those calls.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>arm construction</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>gte-reranker-modernbert-base, seconds</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>Encoding time of gte-reranker-modernbert-base for the index.</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>seconds</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D55"/>
+  <autoFilter ref="A1:D56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
a model call's time is its answering try: the seconds of failed tries out of the call, the question and the run
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finished_data/grag-data.xlsx
+++ b/finished_data/grag-data.xlsx
@@ -8681,10 +8681,10 @@
         <v>0.06868749996647239</v>
       </c>
       <c r="W95" t="n">
-        <v>7.397324400022626</v>
+        <v>6.397227000212297</v>
       </c>
       <c r="X95" t="n">
-        <v>7.469659899827093</v>
+        <v>6.469562500016764</v>
       </c>
       <c r="AB95" t="n">
         <v>22681</v>
@@ -8766,10 +8766,10 @@
         <v>0.1053286001551896</v>
       </c>
       <c r="W96" t="n">
-        <v>8.634245800087228</v>
+        <v>7.633794300025329</v>
       </c>
       <c r="X96" t="n">
-        <v>8.743650400079787</v>
+        <v>7.743198900017887</v>
       </c>
       <c r="AB96" t="n">
         <v>22680</v>
@@ -19512,7 +19512,7 @@
         <v>1.725375100504607</v>
       </c>
       <c r="U210" t="n">
-        <v>12.67415299965069</v>
+        <v>8.987940199673176</v>
       </c>
       <c r="V210" t="n">
         <v>2.321429099887609</v>
@@ -19521,7 +19521,7 @@
         <v>4.968859800137579</v>
       </c>
       <c r="X210" t="n">
-        <v>21.69193159975111</v>
+        <v>18.0057187997736</v>
       </c>
       <c r="Y210" t="n">
         <v>2060</v>
@@ -28379,7 +28379,7 @@
         <v>2.359066299628466</v>
       </c>
       <c r="U296" t="n">
-        <v>24.59212730033323</v>
+        <v>10.31776810018346</v>
       </c>
       <c r="V296" t="n">
         <v>1.303002000320703</v>
@@ -28388,7 +28388,7 @@
         <v>9.826243599876761</v>
       </c>
       <c r="X296" t="n">
-        <v>38.08309690002352</v>
+        <v>23.80873769987375</v>
       </c>
       <c r="Y296" t="n">
         <v>2067</v>
@@ -29052,13 +29052,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>682.8234252999537</v>
+        <v>680.8228764000814</v>
       </c>
       <c r="C10" t="n">
         <v>901.5495188999921</v>
       </c>
       <c r="D10" t="n">
-        <v>2631.523206799757</v>
+        <v>2613.562634799629</v>
       </c>
     </row>
     <row r="11">
@@ -29394,7 +29394,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>13.55906191201415</v>
+        <v>13.37945619201288</v>
       </c>
     </row>
     <row r="33">
@@ -29417,7 +29417,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>6.749374916995875</v>
+        <v>6.729369427997153</v>
       </c>
       <c r="C34" t="n">
         <v>8.107556761973537</v>
@@ -29433,13 +29433,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>6.787730676007922</v>
+        <v>6.767725187009201</v>
       </c>
       <c r="C35" t="n">
         <v>8.667278056973592</v>
       </c>
       <c r="D35" t="n">
-        <v>26.05431466102134</v>
+        <v>25.87470894102007</v>
       </c>
     </row>
     <row r="36">
@@ -30230,7 +30230,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Time of the interpreter call: the answer model, called before retrieval. Artefact only.</t>
+          <t>Time of the interpreter call's answering try: the answer model, called before retrieval. Artefact only.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -30274,7 +30274,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Time of the answer model call.</t>
+          <t>Time of the answer model call's answering try.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -30296,7 +30296,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Time of all steps for the question, to the answer.</t>
+          <t>Time of all steps for the question, to the answer, without failed tries of model calls.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -30504,7 +30504,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Time of the run over the 100 questions.</t>
+          <t>Time of the run over the 100 questions, without failed tries of model calls.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">

</xml_diff>

<commit_message>
export: characters of retrieved context per question (retrieved_context_characters)
</commit_message>
<xml_diff>
--- a/finished_data/grag-data.xlsx
+++ b/finished_data/grag-data.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="key" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'results'!$A$1:$AC$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'results'!$A$1:$AD$301</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'arm construction'!$A$1:$D$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC301"/>
+  <dimension ref="A1:AD301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -454,8 +454,9 @@
     <col width="23" customWidth="1" min="25" max="25"/>
     <col width="24" customWidth="1" min="26" max="26"/>
     <col width="24" customWidth="1" min="27" max="27"/>
-    <col width="18" customWidth="1" min="28" max="28"/>
-    <col width="19" customWidth="1" min="29" max="29"/>
+    <col width="30" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="19" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -596,10 +597,15 @@
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
+          <t>retrieved_context_characters</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
           <t>answer_tokens_in</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>answer_tokens_out</t>
         </is>
@@ -683,9 +689,12 @@
         <v>5.246650699991733</v>
       </c>
       <c r="AB2" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC2" t="n">
         <v>22680</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AD2" t="n">
         <v>171</v>
       </c>
     </row>
@@ -767,9 +776,12 @@
         <v>5.39425399992615</v>
       </c>
       <c r="AB3" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC3" t="n">
         <v>23825</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AD3" t="n">
         <v>200</v>
       </c>
     </row>
@@ -851,9 +863,12 @@
         <v>4.419108100002632</v>
       </c>
       <c r="AB4" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC4" t="n">
         <v>22891</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AD4" t="n">
         <v>127</v>
       </c>
     </row>
@@ -938,9 +953,12 @@
         <v>8.19805010012351</v>
       </c>
       <c r="AB5" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC5" t="n">
         <v>29426</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AD5" t="n">
         <v>427</v>
       </c>
     </row>
@@ -1029,9 +1047,12 @@
         <v>9.131861000088975</v>
       </c>
       <c r="AB6" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC6" t="n">
         <v>23003</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AD6" t="n">
         <v>489</v>
       </c>
     </row>
@@ -1116,9 +1137,12 @@
         <v>6.152991499984637</v>
       </c>
       <c r="AB7" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC7" t="n">
         <v>29121</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AD7" t="n">
         <v>282</v>
       </c>
     </row>
@@ -1200,9 +1224,12 @@
         <v>5.124460299964994</v>
       </c>
       <c r="AB8" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC8" t="n">
         <v>23504</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AD8" t="n">
         <v>198</v>
       </c>
     </row>
@@ -1285,9 +1312,12 @@
         <v>8.036565100075677</v>
       </c>
       <c r="AB9" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC9" t="n">
         <v>24534</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AD9" t="n">
         <v>295</v>
       </c>
     </row>
@@ -1369,9 +1399,12 @@
         <v>5.113492399919778</v>
       </c>
       <c r="AB10" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC10" t="n">
         <v>23513</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AD10" t="n">
         <v>173</v>
       </c>
     </row>
@@ -1459,9 +1492,12 @@
         <v>11.64250219985843</v>
       </c>
       <c r="AB11" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC11" t="n">
         <v>26721</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AD11" t="n">
         <v>731</v>
       </c>
     </row>
@@ -1549,9 +1585,12 @@
         <v>13.43550999998115</v>
       </c>
       <c r="AB12" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC12" t="n">
         <v>29873</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AD12" t="n">
         <v>970</v>
       </c>
     </row>
@@ -1633,9 +1672,12 @@
         <v>5.963001300115138</v>
       </c>
       <c r="AB13" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC13" t="n">
         <v>24726</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="AD13" t="n">
         <v>264</v>
       </c>
     </row>
@@ -1717,9 +1759,12 @@
         <v>4.615674200002104</v>
       </c>
       <c r="AB14" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC14" t="n">
         <v>27637</v>
       </c>
-      <c r="AC14" t="n">
+      <c r="AD14" t="n">
         <v>110</v>
       </c>
     </row>
@@ -1809,9 +1854,12 @@
         <v>8.99069569981657</v>
       </c>
       <c r="AB15" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC15" t="n">
         <v>28327</v>
       </c>
-      <c r="AC15" t="n">
+      <c r="AD15" t="n">
         <v>474</v>
       </c>
     </row>
@@ -1898,9 +1946,12 @@
         <v>8.592069299891591</v>
       </c>
       <c r="AB16" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC16" t="n">
         <v>24804</v>
       </c>
-      <c r="AC16" t="n">
+      <c r="AD16" t="n">
         <v>493</v>
       </c>
     </row>
@@ -1982,9 +2033,12 @@
         <v>5.270493300165981</v>
       </c>
       <c r="AB17" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC17" t="n">
         <v>24065</v>
       </c>
-      <c r="AC17" t="n">
+      <c r="AD17" t="n">
         <v>224</v>
       </c>
     </row>
@@ -2066,9 +2120,12 @@
         <v>6.086556000169367</v>
       </c>
       <c r="AB18" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC18" t="n">
         <v>26704</v>
       </c>
-      <c r="AC18" t="n">
+      <c r="AD18" t="n">
         <v>275</v>
       </c>
     </row>
@@ -2150,9 +2207,12 @@
         <v>6.084697100101039</v>
       </c>
       <c r="AB19" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC19" t="n">
         <v>22924</v>
       </c>
-      <c r="AC19" t="n">
+      <c r="AD19" t="n">
         <v>291</v>
       </c>
     </row>
@@ -2234,9 +2294,12 @@
         <v>6.674424699973315</v>
       </c>
       <c r="AB20" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC20" t="n">
         <v>25603</v>
       </c>
-      <c r="AC20" t="n">
+      <c r="AD20" t="n">
         <v>295</v>
       </c>
     </row>
@@ -2318,9 +2381,12 @@
         <v>5.194544899975881</v>
       </c>
       <c r="AB21" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC21" t="n">
         <v>28019</v>
       </c>
-      <c r="AC21" t="n">
+      <c r="AD21" t="n">
         <v>124</v>
       </c>
     </row>
@@ -2402,9 +2468,12 @@
         <v>5.967118200147524</v>
       </c>
       <c r="AB22" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC22" t="n">
         <v>23900</v>
       </c>
-      <c r="AC22" t="n">
+      <c r="AD22" t="n">
         <v>227</v>
       </c>
     </row>
@@ -2490,9 +2559,12 @@
         <v>4.775314300088212</v>
       </c>
       <c r="AB23" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC23" t="n">
         <v>22962</v>
       </c>
-      <c r="AC23" t="n">
+      <c r="AD23" t="n">
         <v>187</v>
       </c>
     </row>
@@ -2574,9 +2646,12 @@
         <v>4.178553299978375</v>
       </c>
       <c r="AB24" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC24" t="n">
         <v>29501</v>
       </c>
-      <c r="AC24" t="n">
+      <c r="AD24" t="n">
         <v>109</v>
       </c>
     </row>
@@ -2661,9 +2736,12 @@
         <v>5.532242400106043</v>
       </c>
       <c r="AB25" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC25" t="n">
         <v>24246</v>
       </c>
-      <c r="AC25" t="n">
+      <c r="AD25" t="n">
         <v>243</v>
       </c>
     </row>
@@ -2745,9 +2823,12 @@
         <v>8.853384400019422</v>
       </c>
       <c r="AB26" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC26" t="n">
         <v>28908</v>
       </c>
-      <c r="AC26" t="n">
+      <c r="AD26" t="n">
         <v>469</v>
       </c>
     </row>
@@ -2829,9 +2910,12 @@
         <v>4.613873200025409</v>
       </c>
       <c r="AB27" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC27" t="n">
         <v>22647</v>
       </c>
-      <c r="AC27" t="n">
+      <c r="AD27" t="n">
         <v>110</v>
       </c>
     </row>
@@ -2917,9 +3001,12 @@
         <v>8.587901300052181</v>
       </c>
       <c r="AB28" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC28" t="n">
         <v>26486</v>
       </c>
-      <c r="AC28" t="n">
+      <c r="AD28" t="n">
         <v>435</v>
       </c>
     </row>
@@ -3001,9 +3088,12 @@
         <v>4.33954509999603</v>
       </c>
       <c r="AB29" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC29" t="n">
         <v>25605</v>
       </c>
-      <c r="AC29" t="n">
+      <c r="AD29" t="n">
         <v>136</v>
       </c>
     </row>
@@ -3089,9 +3179,12 @@
         <v>5.147288099862635</v>
       </c>
       <c r="AB30" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC30" t="n">
         <v>23716</v>
       </c>
-      <c r="AC30" t="n">
+      <c r="AD30" t="n">
         <v>242</v>
       </c>
     </row>
@@ -3175,9 +3268,12 @@
         <v>6.78785640001297</v>
       </c>
       <c r="AB31" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC31" t="n">
         <v>24202</v>
       </c>
-      <c r="AC31" t="n">
+      <c r="AD31" t="n">
         <v>364</v>
       </c>
     </row>
@@ -3265,9 +3361,12 @@
         <v>10.12143489997834</v>
       </c>
       <c r="AB32" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC32" t="n">
         <v>26691</v>
       </c>
-      <c r="AC32" t="n">
+      <c r="AD32" t="n">
         <v>578</v>
       </c>
     </row>
@@ -3349,9 +3448,12 @@
         <v>6.647219700040296</v>
       </c>
       <c r="AB33" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC33" t="n">
         <v>25032</v>
       </c>
-      <c r="AC33" t="n">
+      <c r="AD33" t="n">
         <v>316</v>
       </c>
     </row>
@@ -3436,9 +3538,12 @@
         <v>7.608983700163662</v>
       </c>
       <c r="AB34" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC34" t="n">
         <v>23565</v>
       </c>
-      <c r="AC34" t="n">
+      <c r="AD34" t="n">
         <v>384</v>
       </c>
     </row>
@@ -3520,9 +3625,12 @@
         <v>4.589931899914518</v>
       </c>
       <c r="AB35" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC35" t="n">
         <v>27793</v>
       </c>
-      <c r="AC35" t="n">
+      <c r="AD35" t="n">
         <v>173</v>
       </c>
     </row>
@@ -3607,9 +3715,12 @@
         <v>5.868815600173548</v>
       </c>
       <c r="AB36" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC36" t="n">
         <v>28368</v>
       </c>
-      <c r="AC36" t="n">
+      <c r="AD36" t="n">
         <v>237</v>
       </c>
     </row>
@@ -3701,9 +3812,12 @@
         <v>14.89762439997867</v>
       </c>
       <c r="AB37" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC37" t="n">
         <v>30608</v>
       </c>
-      <c r="AC37" t="n">
+      <c r="AD37" t="n">
         <v>1023</v>
       </c>
     </row>
@@ -3787,9 +3901,12 @@
         <v>6.417497299844399</v>
       </c>
       <c r="AB38" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC38" t="n">
         <v>25789</v>
       </c>
-      <c r="AC38" t="n">
+      <c r="AD38" t="n">
         <v>263</v>
       </c>
     </row>
@@ -3871,9 +3988,12 @@
         <v>6.61693839984946</v>
       </c>
       <c r="AB39" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC39" t="n">
         <v>22901</v>
       </c>
-      <c r="AC39" t="n">
+      <c r="AD39" t="n">
         <v>275</v>
       </c>
     </row>
@@ -3955,9 +4075,12 @@
         <v>9.978571400046349</v>
       </c>
       <c r="AB40" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC40" t="n">
         <v>25175</v>
       </c>
-      <c r="AC40" t="n">
+      <c r="AD40" t="n">
         <v>648</v>
       </c>
     </row>
@@ -4039,9 +4162,12 @@
         <v>5.548226200044155</v>
       </c>
       <c r="AB41" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC41" t="n">
         <v>25991</v>
       </c>
-      <c r="AC41" t="n">
+      <c r="AD41" t="n">
         <v>218</v>
       </c>
     </row>
@@ -4125,9 +4251,12 @@
         <v>5.453348100185394</v>
       </c>
       <c r="AB42" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC42" t="n">
         <v>27925</v>
       </c>
-      <c r="AC42" t="n">
+      <c r="AD42" t="n">
         <v>220</v>
       </c>
     </row>
@@ -4209,9 +4338,12 @@
         <v>5.11244810000062</v>
       </c>
       <c r="AB43" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC43" t="n">
         <v>22811</v>
       </c>
-      <c r="AC43" t="n">
+      <c r="AD43" t="n">
         <v>193</v>
       </c>
     </row>
@@ -4297,9 +4429,12 @@
         <v>9.034127800026909</v>
       </c>
       <c r="AB44" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC44" t="n">
         <v>23783</v>
       </c>
-      <c r="AC44" t="n">
+      <c r="AD44" t="n">
         <v>473</v>
       </c>
     </row>
@@ -4381,9 +4516,12 @@
         <v>5.94153490010649</v>
       </c>
       <c r="AB45" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC45" t="n">
         <v>27835</v>
       </c>
-      <c r="AC45" t="n">
+      <c r="AD45" t="n">
         <v>247</v>
       </c>
     </row>
@@ -4468,9 +4606,12 @@
         <v>6.45311599993147</v>
       </c>
       <c r="AB46" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC46" t="n">
         <v>24456</v>
       </c>
-      <c r="AC46" t="n">
+      <c r="AD46" t="n">
         <v>361</v>
       </c>
     </row>
@@ -4557,9 +4698,12 @@
         <v>8.547711699968204</v>
       </c>
       <c r="AB47" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC47" t="n">
         <v>24536</v>
       </c>
-      <c r="AC47" t="n">
+      <c r="AD47" t="n">
         <v>459</v>
       </c>
     </row>
@@ -4642,9 +4786,12 @@
         <v>5.524571900023147</v>
       </c>
       <c r="AB48" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC48" t="n">
         <v>23752</v>
       </c>
-      <c r="AC48" t="n">
+      <c r="AD48" t="n">
         <v>270</v>
       </c>
     </row>
@@ -4726,9 +4873,12 @@
         <v>7.642424399964511</v>
       </c>
       <c r="AB49" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC49" t="n">
         <v>30651</v>
       </c>
-      <c r="AC49" t="n">
+      <c r="AD49" t="n">
         <v>426</v>
       </c>
     </row>
@@ -4814,9 +4964,12 @@
         <v>7.258854300016537</v>
       </c>
       <c r="AB50" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC50" t="n">
         <v>24005</v>
       </c>
-      <c r="AC50" t="n">
+      <c r="AD50" t="n">
         <v>371</v>
       </c>
     </row>
@@ -4901,9 +5054,12 @@
         <v>9.109107399825007</v>
       </c>
       <c r="AB51" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC51" t="n">
         <v>23283</v>
       </c>
-      <c r="AC51" t="n">
+      <c r="AD51" t="n">
         <v>518</v>
       </c>
     </row>
@@ -4991,9 +5147,12 @@
         <v>8.036057499935851</v>
       </c>
       <c r="AB52" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC52" t="n">
         <v>27375</v>
       </c>
-      <c r="AC52" t="n">
+      <c r="AD52" t="n">
         <v>470</v>
       </c>
     </row>
@@ -5080,9 +5239,12 @@
         <v>8.817925299983472</v>
       </c>
       <c r="AB53" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC53" t="n">
         <v>24347</v>
       </c>
-      <c r="AC53" t="n">
+      <c r="AD53" t="n">
         <v>537</v>
       </c>
     </row>
@@ -5168,9 +5330,12 @@
         <v>9.227018499979749</v>
       </c>
       <c r="AB54" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC54" t="n">
         <v>28872</v>
       </c>
-      <c r="AC54" t="n">
+      <c r="AD54" t="n">
         <v>472</v>
       </c>
     </row>
@@ -5254,9 +5419,12 @@
         <v>6.274000300094485</v>
       </c>
       <c r="AB55" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC55" t="n">
         <v>35272</v>
       </c>
-      <c r="AC55" t="n">
+      <c r="AD55" t="n">
         <v>267</v>
       </c>
     </row>
@@ -5338,9 +5506,12 @@
         <v>4.577051399974152</v>
       </c>
       <c r="AB56" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC56" t="n">
         <v>26450</v>
       </c>
-      <c r="AC56" t="n">
+      <c r="AD56" t="n">
         <v>170</v>
       </c>
     </row>
@@ -5425,9 +5596,12 @@
         <v>6.299022200051695</v>
       </c>
       <c r="AB57" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC57" t="n">
         <v>25975</v>
       </c>
-      <c r="AC57" t="n">
+      <c r="AD57" t="n">
         <v>375</v>
       </c>
     </row>
@@ -5516,9 +5690,12 @@
         <v>8.925569200189784</v>
       </c>
       <c r="AB58" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC58" t="n">
         <v>24493</v>
       </c>
-      <c r="AC58" t="n">
+      <c r="AD58" t="n">
         <v>563</v>
       </c>
     </row>
@@ -5600,9 +5777,12 @@
         <v>5.407248700037599</v>
       </c>
       <c r="AB59" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC59" t="n">
         <v>24286</v>
       </c>
-      <c r="AC59" t="n">
+      <c r="AD59" t="n">
         <v>206</v>
       </c>
     </row>
@@ -5688,9 +5868,12 @@
         <v>6.101434899959713</v>
       </c>
       <c r="AB60" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC60" t="n">
         <v>23378</v>
       </c>
-      <c r="AC60" t="n">
+      <c r="AD60" t="n">
         <v>322</v>
       </c>
     </row>
@@ -5777,9 +5960,12 @@
         <v>11.67624790011905</v>
       </c>
       <c r="AB61" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC61" t="n">
         <v>31653</v>
       </c>
-      <c r="AC61" t="n">
+      <c r="AD61" t="n">
         <v>731</v>
       </c>
     </row>
@@ -5861,9 +6047,12 @@
         <v>4.606331200106069</v>
       </c>
       <c r="AB62" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC62" t="n">
         <v>35141</v>
       </c>
-      <c r="AC62" t="n">
+      <c r="AD62" t="n">
         <v>138</v>
       </c>
     </row>
@@ -5945,9 +6134,12 @@
         <v>5.460378800053149</v>
       </c>
       <c r="AB63" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC63" t="n">
         <v>34609</v>
       </c>
-      <c r="AC63" t="n">
+      <c r="AD63" t="n">
         <v>218</v>
       </c>
     </row>
@@ -6032,9 +6224,12 @@
         <v>8.161358300130814</v>
       </c>
       <c r="AB64" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC64" t="n">
         <v>28440</v>
       </c>
-      <c r="AC64" t="n">
+      <c r="AD64" t="n">
         <v>407</v>
       </c>
     </row>
@@ -6119,9 +6314,12 @@
         <v>8.015652699861676</v>
       </c>
       <c r="AB65" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC65" t="n">
         <v>27662</v>
       </c>
-      <c r="AC65" t="n">
+      <c r="AD65" t="n">
         <v>473</v>
       </c>
     </row>
@@ -6203,9 +6401,12 @@
         <v>4.910263899946585</v>
       </c>
       <c r="AB66" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC66" t="n">
         <v>26558</v>
       </c>
-      <c r="AC66" t="n">
+      <c r="AD66" t="n">
         <v>153</v>
       </c>
     </row>
@@ -6287,9 +6488,12 @@
         <v>5.234396300045773</v>
       </c>
       <c r="AB67" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC67" t="n">
         <v>23184</v>
       </c>
-      <c r="AC67" t="n">
+      <c r="AD67" t="n">
         <v>271</v>
       </c>
     </row>
@@ -6375,9 +6579,12 @@
         <v>7.415566900046542</v>
       </c>
       <c r="AB68" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC68" t="n">
         <v>35151</v>
       </c>
-      <c r="AC68" t="n">
+      <c r="AD68" t="n">
         <v>350</v>
       </c>
     </row>
@@ -6462,9 +6669,12 @@
         <v>8.168236099882051</v>
       </c>
       <c r="AB69" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC69" t="n">
         <v>26196</v>
       </c>
-      <c r="AC69" t="n">
+      <c r="AD69" t="n">
         <v>422</v>
       </c>
     </row>
@@ -6554,9 +6764,12 @@
         <v>9.444058800116181</v>
       </c>
       <c r="AB70" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC70" t="n">
         <v>26228</v>
       </c>
-      <c r="AC70" t="n">
+      <c r="AD70" t="n">
         <v>613</v>
       </c>
     </row>
@@ -6640,9 +6853,12 @@
         <v>7.954675500048324</v>
       </c>
       <c r="AB71" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC71" t="n">
         <v>26973</v>
       </c>
-      <c r="AC71" t="n">
+      <c r="AD71" t="n">
         <v>434</v>
       </c>
     </row>
@@ -6724,9 +6940,12 @@
         <v>5.264079899992794</v>
       </c>
       <c r="AB72" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC72" t="n">
         <v>26441</v>
       </c>
-      <c r="AC72" t="n">
+      <c r="AD72" t="n">
         <v>202</v>
       </c>
     </row>
@@ -6808,9 +7027,12 @@
         <v>4.288960200035945</v>
       </c>
       <c r="AB73" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC73" t="n">
         <v>32192</v>
       </c>
-      <c r="AC73" t="n">
+      <c r="AD73" t="n">
         <v>126</v>
       </c>
     </row>
@@ -6894,9 +7116,12 @@
         <v>9.216729399980977</v>
       </c>
       <c r="AB74" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC74" t="n">
         <v>24856</v>
       </c>
-      <c r="AC74" t="n">
+      <c r="AD74" t="n">
         <v>572</v>
       </c>
     </row>
@@ -6983,9 +7208,12 @@
         <v>7.822610500035807</v>
       </c>
       <c r="AB75" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC75" t="n">
         <v>27981</v>
       </c>
-      <c r="AC75" t="n">
+      <c r="AD75" t="n">
         <v>409</v>
       </c>
     </row>
@@ -7076,9 +7304,12 @@
         <v>9.938860400114208</v>
       </c>
       <c r="AB76" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC76" t="n">
         <v>35271</v>
       </c>
-      <c r="AC76" t="n">
+      <c r="AD76" t="n">
         <v>567</v>
       </c>
     </row>
@@ -7160,9 +7391,12 @@
         <v>6.054761999985203</v>
       </c>
       <c r="AB77" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC77" t="n">
         <v>26450</v>
       </c>
-      <c r="AC77" t="n">
+      <c r="AD77" t="n">
         <v>321</v>
       </c>
     </row>
@@ -7244,9 +7478,12 @@
         <v>4.5416979000438</v>
       </c>
       <c r="AB78" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC78" t="n">
         <v>26322</v>
       </c>
-      <c r="AC78" t="n">
+      <c r="AD78" t="n">
         <v>139</v>
       </c>
     </row>
@@ -7328,9 +7565,12 @@
         <v>4.505794700002298</v>
       </c>
       <c r="AB79" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC79" t="n">
         <v>26084</v>
       </c>
-      <c r="AC79" t="n">
+      <c r="AD79" t="n">
         <v>227</v>
       </c>
     </row>
@@ -7412,9 +7652,12 @@
         <v>4.986567600164562</v>
       </c>
       <c r="AB80" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC80" t="n">
         <v>25355</v>
       </c>
-      <c r="AC80" t="n">
+      <c r="AD80" t="n">
         <v>181</v>
       </c>
     </row>
@@ -7503,9 +7746,12 @@
         <v>10.33759879996069</v>
       </c>
       <c r="AB81" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC81" t="n">
         <v>29734</v>
       </c>
-      <c r="AC81" t="n">
+      <c r="AD81" t="n">
         <v>662</v>
       </c>
     </row>
@@ -7591,9 +7837,12 @@
         <v>7.185228400165215</v>
       </c>
       <c r="AB82" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC82" t="n">
         <v>25734</v>
       </c>
-      <c r="AC82" t="n">
+      <c r="AD82" t="n">
         <v>334</v>
       </c>
     </row>
@@ -7675,9 +7924,12 @@
         <v>4.705564099829644</v>
       </c>
       <c r="AB83" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC83" t="n">
         <v>35267</v>
       </c>
-      <c r="AC83" t="n">
+      <c r="AD83" t="n">
         <v>204</v>
       </c>
     </row>
@@ -7763,9 +8015,12 @@
         <v>6.370938299922273</v>
       </c>
       <c r="AB84" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC84" t="n">
         <v>27568</v>
       </c>
-      <c r="AC84" t="n">
+      <c r="AD84" t="n">
         <v>331</v>
       </c>
     </row>
@@ -7847,9 +8102,12 @@
         <v>3.971278900047764</v>
       </c>
       <c r="AB85" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC85" t="n">
         <v>26408</v>
       </c>
-      <c r="AC85" t="n">
+      <c r="AD85" t="n">
         <v>97</v>
       </c>
     </row>
@@ -7931,9 +8189,12 @@
         <v>5.818028899841011</v>
       </c>
       <c r="AB86" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC86" t="n">
         <v>26443</v>
       </c>
-      <c r="AC86" t="n">
+      <c r="AD86" t="n">
         <v>279</v>
       </c>
     </row>
@@ -8015,9 +8276,12 @@
         <v>6.360301200067624</v>
       </c>
       <c r="AB87" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC87" t="n">
         <v>35270</v>
       </c>
-      <c r="AC87" t="n">
+      <c r="AD87" t="n">
         <v>262</v>
       </c>
     </row>
@@ -8099,9 +8363,12 @@
         <v>4.519596199970692</v>
       </c>
       <c r="AB88" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC88" t="n">
         <v>26351</v>
       </c>
-      <c r="AC88" t="n">
+      <c r="AD88" t="n">
         <v>112</v>
       </c>
     </row>
@@ -8183,9 +8450,12 @@
         <v>4.71104529988952</v>
       </c>
       <c r="AB89" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC89" t="n">
         <v>26350</v>
       </c>
-      <c r="AC89" t="n">
+      <c r="AD89" t="n">
         <v>174</v>
       </c>
     </row>
@@ -8267,9 +8537,12 @@
         <v>4.244742799783126</v>
       </c>
       <c r="AB90" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC90" t="n">
         <v>23437</v>
       </c>
-      <c r="AC90" t="n">
+      <c r="AD90" t="n">
         <v>109</v>
       </c>
     </row>
@@ -8351,9 +8624,12 @@
         <v>5.585942599922419</v>
       </c>
       <c r="AB91" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC91" t="n">
         <v>23003</v>
       </c>
-      <c r="AC91" t="n">
+      <c r="AD91" t="n">
         <v>181</v>
       </c>
     </row>
@@ -8435,9 +8711,12 @@
         <v>5.787526100175455</v>
       </c>
       <c r="AB92" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC92" t="n">
         <v>23478</v>
       </c>
-      <c r="AC92" t="n">
+      <c r="AD92" t="n">
         <v>217</v>
       </c>
     </row>
@@ -8519,9 +8798,12 @@
         <v>5.285540499957278</v>
       </c>
       <c r="AB93" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC93" t="n">
         <v>22679</v>
       </c>
-      <c r="AC93" t="n">
+      <c r="AD93" t="n">
         <v>192</v>
       </c>
     </row>
@@ -8603,9 +8885,12 @@
         <v>6.118239900097251</v>
       </c>
       <c r="AB94" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC94" t="n">
         <v>23942</v>
       </c>
-      <c r="AC94" t="n">
+      <c r="AD94" t="n">
         <v>245</v>
       </c>
     </row>
@@ -8687,9 +8972,12 @@
         <v>6.469562500016764</v>
       </c>
       <c r="AB95" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC95" t="n">
         <v>22681</v>
       </c>
-      <c r="AC95" t="n">
+      <c r="AD95" t="n">
         <v>100</v>
       </c>
     </row>
@@ -8772,9 +9060,12 @@
         <v>7.743198900017887</v>
       </c>
       <c r="AB96" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC96" t="n">
         <v>22680</v>
       </c>
-      <c r="AC96" t="n">
+      <c r="AD96" t="n">
         <v>165</v>
       </c>
     </row>
@@ -8856,9 +9147,12 @@
         <v>8.903144199866802</v>
       </c>
       <c r="AB97" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC97" t="n">
         <v>23735</v>
       </c>
-      <c r="AC97" t="n">
+      <c r="AD97" t="n">
         <v>316</v>
       </c>
     </row>
@@ -8940,9 +9234,12 @@
         <v>5.333889700006694</v>
       </c>
       <c r="AB98" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC98" t="n">
         <v>22888</v>
       </c>
-      <c r="AC98" t="n">
+      <c r="AD98" t="n">
         <v>121</v>
       </c>
     </row>
@@ -9024,9 +9321,12 @@
         <v>6.780955800088122</v>
       </c>
       <c r="AB99" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC99" t="n">
         <v>22889</v>
       </c>
-      <c r="AC99" t="n">
+      <c r="AD99" t="n">
         <v>190</v>
       </c>
     </row>
@@ -9110,9 +9410,12 @@
         <v>6.770060000009835</v>
       </c>
       <c r="AB100" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC100" t="n">
         <v>22683</v>
       </c>
-      <c r="AC100" t="n">
+      <c r="AD100" t="n">
         <v>210</v>
       </c>
     </row>
@@ -9194,9 +9497,12 @@
         <v>5.914411899866536</v>
       </c>
       <c r="AB101" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC101" t="n">
         <v>22681</v>
       </c>
-      <c r="AC101" t="n">
+      <c r="AD101" t="n">
         <v>161</v>
       </c>
     </row>
@@ -9303,9 +9609,12 @@
         <v>24</v>
       </c>
       <c r="AB102" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC102" t="n">
         <v>30684</v>
       </c>
-      <c r="AC102" t="n">
+      <c r="AD102" t="n">
         <v>1095</v>
       </c>
     </row>
@@ -9397,9 +9706,12 @@
         <v>22</v>
       </c>
       <c r="AB103" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC103" t="n">
         <v>25646</v>
       </c>
-      <c r="AC103" t="n">
+      <c r="AD103" t="n">
         <v>213</v>
       </c>
     </row>
@@ -9487,9 +9799,12 @@
         <v>23</v>
       </c>
       <c r="AB104" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC104" t="n">
         <v>34049</v>
       </c>
-      <c r="AC104" t="n">
+      <c r="AD104" t="n">
         <v>124</v>
       </c>
     </row>
@@ -9578,9 +9893,12 @@
         <v>26</v>
       </c>
       <c r="AB105" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC105" t="n">
         <v>32885</v>
       </c>
-      <c r="AC105" t="n">
+      <c r="AD105" t="n">
         <v>209</v>
       </c>
     </row>
@@ -9669,9 +9987,12 @@
         <v>22</v>
       </c>
       <c r="AB106" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC106" t="n">
         <v>25777</v>
       </c>
-      <c r="AC106" t="n">
+      <c r="AD106" t="n">
         <v>343</v>
       </c>
     </row>
@@ -9761,9 +10082,12 @@
         <v>24</v>
       </c>
       <c r="AB107" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC107" t="n">
         <v>32021</v>
       </c>
-      <c r="AC107" t="n">
+      <c r="AD107" t="n">
         <v>266</v>
       </c>
     </row>
@@ -9854,9 +10178,12 @@
         <v>31</v>
       </c>
       <c r="AB108" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC108" t="n">
         <v>32026</v>
       </c>
-      <c r="AC108" t="n">
+      <c r="AD108" t="n">
         <v>373</v>
       </c>
     </row>
@@ -9944,9 +10271,12 @@
         <v>22</v>
       </c>
       <c r="AB109" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC109" t="n">
         <v>25903</v>
       </c>
-      <c r="AC109" t="n">
+      <c r="AD109" t="n">
         <v>177</v>
       </c>
     </row>
@@ -10034,9 +10364,12 @@
         <v>19</v>
       </c>
       <c r="AB110" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC110" t="n">
         <v>31236</v>
       </c>
-      <c r="AC110" t="n">
+      <c r="AD110" t="n">
         <v>249</v>
       </c>
     </row>
@@ -10124,9 +10457,12 @@
         <v>19</v>
       </c>
       <c r="AB111" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC111" t="n">
         <v>32690</v>
       </c>
-      <c r="AC111" t="n">
+      <c r="AD111" t="n">
         <v>105</v>
       </c>
     </row>
@@ -10219,9 +10555,12 @@
         <v>30</v>
       </c>
       <c r="AB112" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC112" t="n">
         <v>30783</v>
       </c>
-      <c r="AC112" t="n">
+      <c r="AD112" t="n">
         <v>425</v>
       </c>
     </row>
@@ -10311,9 +10650,12 @@
         <v>17</v>
       </c>
       <c r="AB113" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC113" t="n">
         <v>29591</v>
       </c>
-      <c r="AC113" t="n">
+      <c r="AD113" t="n">
         <v>423</v>
       </c>
     </row>
@@ -10401,9 +10743,12 @@
         <v>19</v>
       </c>
       <c r="AB114" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC114" t="n">
         <v>32854</v>
       </c>
-      <c r="AC114" t="n">
+      <c r="AD114" t="n">
         <v>423</v>
       </c>
     </row>
@@ -10495,9 +10840,12 @@
         <v>17</v>
       </c>
       <c r="AB115" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC115" t="n">
         <v>31383</v>
       </c>
-      <c r="AC115" t="n">
+      <c r="AD115" t="n">
         <v>407</v>
       </c>
     </row>
@@ -10593,9 +10941,12 @@
         <v>21</v>
       </c>
       <c r="AB116" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC116" t="n">
         <v>25591</v>
       </c>
-      <c r="AC116" t="n">
+      <c r="AD116" t="n">
         <v>908</v>
       </c>
     </row>
@@ -10698,9 +11049,12 @@
         <v>22</v>
       </c>
       <c r="AB117" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC117" t="n">
         <v>26122</v>
       </c>
-      <c r="AC117" t="n">
+      <c r="AD117" t="n">
         <v>597</v>
       </c>
     </row>
@@ -10788,9 +11142,12 @@
         <v>18</v>
       </c>
       <c r="AB118" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC118" t="n">
         <v>32870</v>
       </c>
-      <c r="AC118" t="n">
+      <c r="AD118" t="n">
         <v>205</v>
       </c>
     </row>
@@ -10883,9 +11240,12 @@
         <v>24</v>
       </c>
       <c r="AB119" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC119" t="n">
         <v>32838</v>
       </c>
-      <c r="AC119" t="n">
+      <c r="AD119" t="n">
         <v>532</v>
       </c>
     </row>
@@ -10973,9 +11333,12 @@
         <v>22</v>
       </c>
       <c r="AB120" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC120" t="n">
         <v>27106</v>
       </c>
-      <c r="AC120" t="n">
+      <c r="AD120" t="n">
         <v>201</v>
       </c>
     </row>
@@ -11063,9 +11426,12 @@
         <v>17</v>
       </c>
       <c r="AB121" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC121" t="n">
         <v>31680</v>
       </c>
-      <c r="AC121" t="n">
+      <c r="AD121" t="n">
         <v>98</v>
       </c>
     </row>
@@ -11160,9 +11526,12 @@
         <v>21</v>
       </c>
       <c r="AB122" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC122" t="n">
         <v>25745</v>
       </c>
-      <c r="AC122" t="n">
+      <c r="AD122" t="n">
         <v>254</v>
       </c>
     </row>
@@ -11252,9 +11621,12 @@
         <v>15</v>
       </c>
       <c r="AB123" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC123" t="n">
         <v>24925</v>
       </c>
-      <c r="AC123" t="n">
+      <c r="AD123" t="n">
         <v>338</v>
       </c>
     </row>
@@ -11342,9 +11714,12 @@
         <v>18</v>
       </c>
       <c r="AB124" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC124" t="n">
         <v>32308</v>
       </c>
-      <c r="AC124" t="n">
+      <c r="AD124" t="n">
         <v>363</v>
       </c>
     </row>
@@ -11445,9 +11820,12 @@
         <v>14</v>
       </c>
       <c r="AB125" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC125" t="n">
         <v>26016</v>
       </c>
-      <c r="AC125" t="n">
+      <c r="AD125" t="n">
         <v>470</v>
       </c>
     </row>
@@ -11535,9 +11913,12 @@
         <v>20</v>
       </c>
       <c r="AB126" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC126" t="n">
         <v>32361</v>
       </c>
-      <c r="AC126" t="n">
+      <c r="AD126" t="n">
         <v>128</v>
       </c>
     </row>
@@ -11630,9 +12011,12 @@
         <v>26</v>
       </c>
       <c r="AB127" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC127" t="n">
         <v>28714</v>
       </c>
-      <c r="AC127" t="n">
+      <c r="AD127" t="n">
         <v>223</v>
       </c>
     </row>
@@ -11728,9 +12112,12 @@
         <v>15</v>
       </c>
       <c r="AB128" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC128" t="n">
         <v>31937</v>
       </c>
-      <c r="AC128" t="n">
+      <c r="AD128" t="n">
         <v>579</v>
       </c>
     </row>
@@ -11818,9 +12205,12 @@
         <v>18</v>
       </c>
       <c r="AB129" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC129" t="n">
         <v>29619</v>
       </c>
-      <c r="AC129" t="n">
+      <c r="AD129" t="n">
         <v>309</v>
       </c>
     </row>
@@ -11911,9 +12301,12 @@
         <v>19</v>
       </c>
       <c r="AB130" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC130" t="n">
         <v>32461</v>
       </c>
-      <c r="AC130" t="n">
+      <c r="AD130" t="n">
         <v>195</v>
       </c>
     </row>
@@ -12006,9 +12399,12 @@
         <v>32</v>
       </c>
       <c r="AB131" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC131" t="n">
         <v>30898</v>
       </c>
-      <c r="AC131" t="n">
+      <c r="AD131" t="n">
         <v>485</v>
       </c>
     </row>
@@ -12102,9 +12498,12 @@
         <v>21</v>
       </c>
       <c r="AB132" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC132" t="n">
         <v>29474</v>
       </c>
-      <c r="AC132" t="n">
+      <c r="AD132" t="n">
         <v>946</v>
       </c>
     </row>
@@ -12192,9 +12591,12 @@
         <v>24</v>
       </c>
       <c r="AB133" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC133" t="n">
         <v>33824</v>
       </c>
-      <c r="AC133" t="n">
+      <c r="AD133" t="n">
         <v>243</v>
       </c>
     </row>
@@ -12291,9 +12693,12 @@
         <v>20</v>
       </c>
       <c r="AB134" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC134" t="n">
         <v>32512</v>
       </c>
-      <c r="AC134" t="n">
+      <c r="AD134" t="n">
         <v>633</v>
       </c>
     </row>
@@ -12386,9 +12791,12 @@
         <v>24</v>
       </c>
       <c r="AB135" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC135" t="n">
         <v>32978</v>
       </c>
-      <c r="AC135" t="n">
+      <c r="AD135" t="n">
         <v>506</v>
       </c>
     </row>
@@ -12479,9 +12887,12 @@
         <v>31</v>
       </c>
       <c r="AB136" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC136" t="n">
         <v>31490</v>
       </c>
-      <c r="AC136" t="n">
+      <c r="AD136" t="n">
         <v>323</v>
       </c>
     </row>
@@ -12576,9 +12987,12 @@
         <v>15</v>
       </c>
       <c r="AB137" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC137" t="n">
         <v>30647</v>
       </c>
-      <c r="AC137" t="n">
+      <c r="AD137" t="n">
         <v>714</v>
       </c>
     </row>
@@ -12673,9 +13087,12 @@
         <v>29</v>
       </c>
       <c r="AB138" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC138" t="n">
         <v>31101</v>
       </c>
-      <c r="AC138" t="n">
+      <c r="AD138" t="n">
         <v>845</v>
       </c>
     </row>
@@ -12768,9 +13185,12 @@
         <v>16</v>
       </c>
       <c r="AB139" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC139" t="n">
         <v>24858</v>
       </c>
-      <c r="AC139" t="n">
+      <c r="AD139" t="n">
         <v>454</v>
       </c>
     </row>
@@ -12884,9 +13304,12 @@
         <v>29</v>
       </c>
       <c r="AB140" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC140" t="n">
         <v>32784</v>
       </c>
-      <c r="AC140" t="n">
+      <c r="AD140" t="n">
         <v>1287</v>
       </c>
     </row>
@@ -12978,9 +13401,12 @@
         <v>20</v>
       </c>
       <c r="AB141" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC141" t="n">
         <v>26673</v>
       </c>
-      <c r="AC141" t="n">
+      <c r="AD141" t="n">
         <v>368</v>
       </c>
     </row>
@@ -13071,9 +13497,12 @@
         <v>34</v>
       </c>
       <c r="AB142" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC142" t="n">
         <v>31440</v>
       </c>
-      <c r="AC142" t="n">
+      <c r="AD142" t="n">
         <v>284</v>
       </c>
     </row>
@@ -13163,9 +13592,12 @@
         <v>17</v>
       </c>
       <c r="AB143" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC143" t="n">
         <v>26656</v>
       </c>
-      <c r="AC143" t="n">
+      <c r="AD143" t="n">
         <v>316</v>
       </c>
     </row>
@@ -13263,9 +13695,12 @@
         <v>18</v>
       </c>
       <c r="AB144" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC144" t="n">
         <v>27977</v>
       </c>
-      <c r="AC144" t="n">
+      <c r="AD144" t="n">
         <v>563</v>
       </c>
     </row>
@@ -13353,9 +13788,12 @@
         <v>24</v>
       </c>
       <c r="AB145" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC145" t="n">
         <v>31277</v>
       </c>
-      <c r="AC145" t="n">
+      <c r="AD145" t="n">
         <v>268</v>
       </c>
     </row>
@@ -13447,9 +13885,12 @@
         <v>21</v>
       </c>
       <c r="AB146" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC146" t="n">
         <v>28703</v>
       </c>
-      <c r="AC146" t="n">
+      <c r="AD146" t="n">
         <v>373</v>
       </c>
     </row>
@@ -13545,9 +13986,12 @@
         <v>18</v>
       </c>
       <c r="AB147" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC147" t="n">
         <v>26073</v>
       </c>
-      <c r="AC147" t="n">
+      <c r="AD147" t="n">
         <v>661</v>
       </c>
     </row>
@@ -13643,9 +14087,12 @@
         <v>28</v>
       </c>
       <c r="AB148" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC148" t="n">
         <v>32300</v>
       </c>
-      <c r="AC148" t="n">
+      <c r="AD148" t="n">
         <v>474</v>
       </c>
     </row>
@@ -13733,9 +14180,12 @@
         <v>20</v>
       </c>
       <c r="AB149" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC149" t="n">
         <v>32590</v>
       </c>
-      <c r="AC149" t="n">
+      <c r="AD149" t="n">
         <v>311</v>
       </c>
     </row>
@@ -13827,9 +14277,12 @@
         <v>33</v>
       </c>
       <c r="AB150" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC150" t="n">
         <v>26341</v>
       </c>
-      <c r="AC150" t="n">
+      <c r="AD150" t="n">
         <v>255</v>
       </c>
     </row>
@@ -13921,9 +14374,12 @@
         <v>40</v>
       </c>
       <c r="AB151" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC151" t="n">
         <v>30954</v>
       </c>
-      <c r="AC151" t="n">
+      <c r="AD151" t="n">
         <v>643</v>
       </c>
     </row>
@@ -14016,9 +14472,12 @@
         <v>15</v>
       </c>
       <c r="AB152" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC152" t="n">
         <v>27759</v>
       </c>
-      <c r="AC152" t="n">
+      <c r="AD152" t="n">
         <v>389</v>
       </c>
     </row>
@@ -14109,9 +14568,12 @@
         <v>41</v>
       </c>
       <c r="AB153" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC153" t="n">
         <v>33154</v>
       </c>
-      <c r="AC153" t="n">
+      <c r="AD153" t="n">
         <v>188</v>
       </c>
     </row>
@@ -14205,9 +14667,12 @@
         <v>28</v>
       </c>
       <c r="AB154" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC154" t="n">
         <v>30563</v>
       </c>
-      <c r="AC154" t="n">
+      <c r="AD154" t="n">
         <v>512</v>
       </c>
     </row>
@@ -14303,9 +14768,12 @@
         <v>21</v>
       </c>
       <c r="AB155" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC155" t="n">
         <v>31424</v>
       </c>
-      <c r="AC155" t="n">
+      <c r="AD155" t="n">
         <v>852</v>
       </c>
     </row>
@@ -14393,9 +14861,12 @@
         <v>19</v>
       </c>
       <c r="AB156" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC156" t="n">
         <v>32543</v>
       </c>
-      <c r="AC156" t="n">
+      <c r="AD156" t="n">
         <v>202</v>
       </c>
     </row>
@@ -14489,9 +14960,12 @@
         <v>17</v>
       </c>
       <c r="AB157" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC157" t="n">
         <v>27161</v>
       </c>
-      <c r="AC157" t="n">
+      <c r="AD157" t="n">
         <v>463</v>
       </c>
     </row>
@@ -14581,9 +15055,12 @@
         <v>25</v>
       </c>
       <c r="AB158" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC158" t="n">
         <v>32200</v>
       </c>
-      <c r="AC158" t="n">
+      <c r="AD158" t="n">
         <v>321</v>
       </c>
     </row>
@@ -14676,9 +15153,12 @@
         <v>19</v>
       </c>
       <c r="AB159" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC159" t="n">
         <v>31007</v>
       </c>
-      <c r="AC159" t="n">
+      <c r="AD159" t="n">
         <v>412</v>
       </c>
     </row>
@@ -14773,9 +15253,12 @@
         <v>19</v>
       </c>
       <c r="AB160" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC160" t="n">
         <v>28426</v>
       </c>
-      <c r="AC160" t="n">
+      <c r="AD160" t="n">
         <v>719</v>
       </c>
     </row>
@@ -14869,9 +15352,12 @@
         <v>27</v>
       </c>
       <c r="AB161" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC161" t="n">
         <v>31136</v>
       </c>
-      <c r="AC161" t="n">
+      <c r="AD161" t="n">
         <v>1119</v>
       </c>
     </row>
@@ -14966,9 +15452,12 @@
         <v>22</v>
       </c>
       <c r="AB162" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC162" t="n">
         <v>32986</v>
       </c>
-      <c r="AC162" t="n">
+      <c r="AD162" t="n">
         <v>553</v>
       </c>
     </row>
@@ -15063,9 +15552,12 @@
         <v>20</v>
       </c>
       <c r="AB163" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC163" t="n">
         <v>30873</v>
       </c>
-      <c r="AC163" t="n">
+      <c r="AD163" t="n">
         <v>625</v>
       </c>
     </row>
@@ -15157,9 +15649,12 @@
         <v>19</v>
       </c>
       <c r="AB164" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC164" t="n">
         <v>28427</v>
       </c>
-      <c r="AC164" t="n">
+      <c r="AD164" t="n">
         <v>322</v>
       </c>
     </row>
@@ -15250,9 +15745,12 @@
         <v>32</v>
       </c>
       <c r="AB165" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC165" t="n">
         <v>31015</v>
       </c>
-      <c r="AC165" t="n">
+      <c r="AD165" t="n">
         <v>277</v>
       </c>
     </row>
@@ -15355,9 +15853,12 @@
         <v>19</v>
       </c>
       <c r="AB166" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC166" t="n">
         <v>30120</v>
       </c>
-      <c r="AC166" t="n">
+      <c r="AD166" t="n">
         <v>489</v>
       </c>
     </row>
@@ -15453,9 +15954,12 @@
         <v>18</v>
       </c>
       <c r="AB167" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC167" t="n">
         <v>25982</v>
       </c>
-      <c r="AC167" t="n">
+      <c r="AD167" t="n">
         <v>556</v>
       </c>
     </row>
@@ -15546,9 +16050,12 @@
         <v>19</v>
       </c>
       <c r="AB168" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC168" t="n">
         <v>31746</v>
       </c>
-      <c r="AC168" t="n">
+      <c r="AD168" t="n">
         <v>561</v>
       </c>
     </row>
@@ -15639,9 +16146,12 @@
         <v>19</v>
       </c>
       <c r="AB169" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC169" t="n">
         <v>27307</v>
       </c>
-      <c r="AC169" t="n">
+      <c r="AD169" t="n">
         <v>437</v>
       </c>
     </row>
@@ -15738,9 +16248,12 @@
         <v>19</v>
       </c>
       <c r="AB170" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC170" t="n">
         <v>28976</v>
       </c>
-      <c r="AC170" t="n">
+      <c r="AD170" t="n">
         <v>852</v>
       </c>
     </row>
@@ -15831,9 +16344,12 @@
         <v>29</v>
       </c>
       <c r="AB171" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC171" t="n">
         <v>30446</v>
       </c>
-      <c r="AC171" t="n">
+      <c r="AD171" t="n">
         <v>613</v>
       </c>
     </row>
@@ -15921,9 +16437,12 @@
         <v>17</v>
       </c>
       <c r="AB172" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC172" t="n">
         <v>31432</v>
       </c>
-      <c r="AC172" t="n">
+      <c r="AD172" t="n">
         <v>179</v>
       </c>
     </row>
@@ -16011,9 +16530,12 @@
         <v>28</v>
       </c>
       <c r="AB173" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC173" t="n">
         <v>33472</v>
       </c>
-      <c r="AC173" t="n">
+      <c r="AD173" t="n">
         <v>217</v>
       </c>
     </row>
@@ -16106,9 +16628,12 @@
         <v>36</v>
       </c>
       <c r="AB174" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC174" t="n">
         <v>30657</v>
       </c>
-      <c r="AC174" t="n">
+      <c r="AD174" t="n">
         <v>736</v>
       </c>
     </row>
@@ -16199,9 +16724,12 @@
         <v>21</v>
       </c>
       <c r="AB175" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC175" t="n">
         <v>29598</v>
       </c>
-      <c r="AC175" t="n">
+      <c r="AD175" t="n">
         <v>473</v>
       </c>
     </row>
@@ -16291,9 +16819,12 @@
         <v>20</v>
       </c>
       <c r="AB176" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC176" t="n">
         <v>33579</v>
       </c>
-      <c r="AC176" t="n">
+      <c r="AD176" t="n">
         <v>212</v>
       </c>
     </row>
@@ -16381,9 +16912,12 @@
         <v>19</v>
       </c>
       <c r="AB177" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC177" t="n">
         <v>31396</v>
       </c>
-      <c r="AC177" t="n">
+      <c r="AD177" t="n">
         <v>172</v>
       </c>
     </row>
@@ -16471,9 +17005,12 @@
         <v>21</v>
       </c>
       <c r="AB178" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC178" t="n">
         <v>31700</v>
       </c>
-      <c r="AC178" t="n">
+      <c r="AD178" t="n">
         <v>110</v>
       </c>
     </row>
@@ -16561,9 +17098,12 @@
         <v>17</v>
       </c>
       <c r="AB179" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC179" t="n">
         <v>32295</v>
       </c>
-      <c r="AC179" t="n">
+      <c r="AD179" t="n">
         <v>207</v>
       </c>
     </row>
@@ -16651,9 +17191,12 @@
         <v>17</v>
       </c>
       <c r="AB180" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC180" t="n">
         <v>31835</v>
       </c>
-      <c r="AC180" t="n">
+      <c r="AD180" t="n">
         <v>258</v>
       </c>
     </row>
@@ -16750,9 +17293,12 @@
         <v>18</v>
       </c>
       <c r="AB181" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC181" t="n">
         <v>27784</v>
       </c>
-      <c r="AC181" t="n">
+      <c r="AD181" t="n">
         <v>781</v>
       </c>
     </row>
@@ -16844,9 +17390,12 @@
         <v>33</v>
       </c>
       <c r="AB182" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC182" t="n">
         <v>30792</v>
       </c>
-      <c r="AC182" t="n">
+      <c r="AD182" t="n">
         <v>819</v>
       </c>
     </row>
@@ -16939,9 +17488,12 @@
         <v>19</v>
       </c>
       <c r="AB183" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC183" t="n">
         <v>31516</v>
       </c>
-      <c r="AC183" t="n">
+      <c r="AD183" t="n">
         <v>455</v>
       </c>
     </row>
@@ -17038,9 +17590,12 @@
         <v>17</v>
       </c>
       <c r="AB184" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC184" t="n">
         <v>27299</v>
       </c>
-      <c r="AC184" t="n">
+      <c r="AD184" t="n">
         <v>540</v>
       </c>
     </row>
@@ -17128,9 +17683,12 @@
         <v>18</v>
       </c>
       <c r="AB185" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC185" t="n">
         <v>31721</v>
       </c>
-      <c r="AC185" t="n">
+      <c r="AD185" t="n">
         <v>235</v>
       </c>
     </row>
@@ -17218,9 +17776,12 @@
         <v>18</v>
       </c>
       <c r="AB186" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC186" t="n">
         <v>30766</v>
       </c>
-      <c r="AC186" t="n">
+      <c r="AD186" t="n">
         <v>177</v>
       </c>
     </row>
@@ -17317,9 +17878,12 @@
         <v>20</v>
       </c>
       <c r="AB187" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC187" t="n">
         <v>31499</v>
       </c>
-      <c r="AC187" t="n">
+      <c r="AD187" t="n">
         <v>803</v>
       </c>
     </row>
@@ -17407,9 +17971,12 @@
         <v>17</v>
       </c>
       <c r="AB188" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC188" t="n">
         <v>32578</v>
       </c>
-      <c r="AC188" t="n">
+      <c r="AD188" t="n">
         <v>303</v>
       </c>
     </row>
@@ -17497,9 +18064,12 @@
         <v>18</v>
       </c>
       <c r="AB189" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC189" t="n">
         <v>32627</v>
       </c>
-      <c r="AC189" t="n">
+      <c r="AD189" t="n">
         <v>263</v>
       </c>
     </row>
@@ -17597,9 +18167,12 @@
         <v>24</v>
       </c>
       <c r="AB190" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC190" t="n">
         <v>31666</v>
       </c>
-      <c r="AC190" t="n">
+      <c r="AD190" t="n">
         <v>811</v>
       </c>
     </row>
@@ -17700,9 +18273,12 @@
         <v>22</v>
       </c>
       <c r="AB191" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC191" t="n">
         <v>26428</v>
       </c>
-      <c r="AC191" t="n">
+      <c r="AD191" t="n">
         <v>487</v>
       </c>
     </row>
@@ -17790,9 +18366,12 @@
         <v>21</v>
       </c>
       <c r="AB192" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC192" t="n">
         <v>33071</v>
       </c>
-      <c r="AC192" t="n">
+      <c r="AD192" t="n">
         <v>124</v>
       </c>
     </row>
@@ -17891,9 +18470,12 @@
         <v>23</v>
       </c>
       <c r="AB193" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC193" t="n">
         <v>26793</v>
       </c>
-      <c r="AC193" t="n">
+      <c r="AD193" t="n">
         <v>480</v>
       </c>
     </row>
@@ -17990,9 +18572,12 @@
         <v>22</v>
       </c>
       <c r="AB194" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC194" t="n">
         <v>25639</v>
       </c>
-      <c r="AC194" t="n">
+      <c r="AD194" t="n">
         <v>380</v>
       </c>
     </row>
@@ -18080,9 +18665,12 @@
         <v>23</v>
       </c>
       <c r="AB195" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC195" t="n">
         <v>29144</v>
       </c>
-      <c r="AC195" t="n">
+      <c r="AD195" t="n">
         <v>335</v>
       </c>
     </row>
@@ -18170,9 +18758,12 @@
         <v>23</v>
       </c>
       <c r="AB196" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC196" t="n">
         <v>28790</v>
       </c>
-      <c r="AC196" t="n">
+      <c r="AD196" t="n">
         <v>204</v>
       </c>
     </row>
@@ -18266,9 +18857,12 @@
         <v>21</v>
       </c>
       <c r="AB197" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC197" t="n">
         <v>26185</v>
       </c>
-      <c r="AC197" t="n">
+      <c r="AD197" t="n">
         <v>231</v>
       </c>
     </row>
@@ -18356,9 +18950,12 @@
         <v>21</v>
       </c>
       <c r="AB198" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC198" t="n">
         <v>32296</v>
       </c>
-      <c r="AC198" t="n">
+      <c r="AD198" t="n">
         <v>163</v>
       </c>
     </row>
@@ -18446,9 +19043,12 @@
         <v>21</v>
       </c>
       <c r="AB199" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC199" t="n">
         <v>31985</v>
       </c>
-      <c r="AC199" t="n">
+      <c r="AD199" t="n">
         <v>131</v>
       </c>
     </row>
@@ -18537,9 +19137,12 @@
         <v>24</v>
       </c>
       <c r="AB200" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC200" t="n">
         <v>29542</v>
       </c>
-      <c r="AC200" t="n">
+      <c r="AD200" t="n">
         <v>397</v>
       </c>
     </row>
@@ -18627,9 +19230,12 @@
         <v>23</v>
       </c>
       <c r="AB201" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC201" t="n">
         <v>29806</v>
       </c>
-      <c r="AC201" t="n">
+      <c r="AD201" t="n">
         <v>426</v>
       </c>
     </row>
@@ -18727,9 +19333,12 @@
         <v>113</v>
       </c>
       <c r="AB202" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC202" t="n">
         <v>30084</v>
       </c>
-      <c r="AC202" t="n">
+      <c r="AD202" t="n">
         <v>359</v>
       </c>
     </row>
@@ -18826,9 +19435,12 @@
         <v>108</v>
       </c>
       <c r="AB203" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC203" t="n">
         <v>32885</v>
       </c>
-      <c r="AC203" t="n">
+      <c r="AD203" t="n">
         <v>224</v>
       </c>
     </row>
@@ -18925,9 +19537,12 @@
         <v>130</v>
       </c>
       <c r="AB204" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC204" t="n">
         <v>34557</v>
       </c>
-      <c r="AC204" t="n">
+      <c r="AD204" t="n">
         <v>122</v>
       </c>
     </row>
@@ -19026,9 +19641,12 @@
         <v>168</v>
       </c>
       <c r="AB205" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC205" t="n">
         <v>33701</v>
       </c>
-      <c r="AC205" t="n">
+      <c r="AD205" t="n">
         <v>242</v>
       </c>
     </row>
@@ -19132,9 +19750,12 @@
         <v>103</v>
       </c>
       <c r="AB206" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC206" t="n">
         <v>31738</v>
       </c>
-      <c r="AC206" t="n">
+      <c r="AD206" t="n">
         <v>510</v>
       </c>
     </row>
@@ -19235,9 +19856,12 @@
         <v>151</v>
       </c>
       <c r="AB207" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC207" t="n">
         <v>33248</v>
       </c>
-      <c r="AC207" t="n">
+      <c r="AD207" t="n">
         <v>360</v>
       </c>
     </row>
@@ -19335,9 +19959,12 @@
         <v>186</v>
       </c>
       <c r="AB208" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC208" t="n">
         <v>34672</v>
       </c>
-      <c r="AC208" t="n">
+      <c r="AD208" t="n">
         <v>331</v>
       </c>
     </row>
@@ -19434,9 +20061,12 @@
         <v>133</v>
       </c>
       <c r="AB209" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC209" t="n">
         <v>31440</v>
       </c>
-      <c r="AC209" t="n">
+      <c r="AD209" t="n">
         <v>176</v>
       </c>
     </row>
@@ -19533,9 +20163,12 @@
         <v>98</v>
       </c>
       <c r="AB210" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC210" t="n">
         <v>32555</v>
       </c>
-      <c r="AC210" t="n">
+      <c r="AD210" t="n">
         <v>144</v>
       </c>
     </row>
@@ -19632,9 +20265,12 @@
         <v>100</v>
       </c>
       <c r="AB211" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC211" t="n">
         <v>33971</v>
       </c>
-      <c r="AC211" t="n">
+      <c r="AD211" t="n">
         <v>90</v>
       </c>
     </row>
@@ -19738,9 +20374,12 @@
         <v>141</v>
       </c>
       <c r="AB212" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC212" t="n">
         <v>32984</v>
       </c>
-      <c r="AC212" t="n">
+      <c r="AD212" t="n">
         <v>510</v>
       </c>
     </row>
@@ -19843,9 +20482,12 @@
         <v>115</v>
       </c>
       <c r="AB213" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC213" t="n">
         <v>30542</v>
       </c>
-      <c r="AC213" t="n">
+      <c r="AD213" t="n">
         <v>360</v>
       </c>
     </row>
@@ -19948,9 +20590,12 @@
         <v>86</v>
       </c>
       <c r="AB214" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC214" t="n">
         <v>34517</v>
       </c>
-      <c r="AC214" t="n">
+      <c r="AD214" t="n">
         <v>619</v>
       </c>
     </row>
@@ -20051,9 +20696,12 @@
         <v>124</v>
       </c>
       <c r="AB215" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC215" t="n">
         <v>32770</v>
       </c>
-      <c r="AC215" t="n">
+      <c r="AD215" t="n">
         <v>364</v>
       </c>
     </row>
@@ -20155,9 +20803,12 @@
         <v>125</v>
       </c>
       <c r="AB216" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC216" t="n">
         <v>30949</v>
       </c>
-      <c r="AC216" t="n">
+      <c r="AD216" t="n">
         <v>532</v>
       </c>
     </row>
@@ -20263,9 +20914,12 @@
         <v>132</v>
       </c>
       <c r="AB217" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC217" t="n">
         <v>32199</v>
       </c>
-      <c r="AC217" t="n">
+      <c r="AD217" t="n">
         <v>322</v>
       </c>
     </row>
@@ -20371,9 +21025,12 @@
         <v>95</v>
       </c>
       <c r="AB218" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC218" t="n">
         <v>34028</v>
       </c>
-      <c r="AC218" t="n">
+      <c r="AD218" t="n">
         <v>615</v>
       </c>
     </row>
@@ -20477,9 +21134,12 @@
         <v>130</v>
       </c>
       <c r="AB219" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC219" t="n">
         <v>32625</v>
       </c>
-      <c r="AC219" t="n">
+      <c r="AD219" t="n">
         <v>441</v>
       </c>
     </row>
@@ -20576,9 +21236,12 @@
         <v>121</v>
       </c>
       <c r="AB220" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC220" t="n">
         <v>33037</v>
       </c>
-      <c r="AC220" t="n">
+      <c r="AD220" t="n">
         <v>152</v>
       </c>
     </row>
@@ -20680,9 +21343,12 @@
         <v>101</v>
       </c>
       <c r="AB221" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC221" t="n">
         <v>33144</v>
       </c>
-      <c r="AC221" t="n">
+      <c r="AD221" t="n">
         <v>335</v>
       </c>
     </row>
@@ -20785,9 +21451,12 @@
         <v>122</v>
       </c>
       <c r="AB222" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC222" t="n">
         <v>31128</v>
       </c>
-      <c r="AC222" t="n">
+      <c r="AD222" t="n">
         <v>364</v>
       </c>
     </row>
@@ -20901,9 +21570,12 @@
         <v>98</v>
       </c>
       <c r="AB223" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC223" t="n">
         <v>31507</v>
       </c>
-      <c r="AC223" t="n">
+      <c r="AD223" t="n">
         <v>700</v>
       </c>
     </row>
@@ -21000,9 +21672,12 @@
         <v>92</v>
       </c>
       <c r="AB224" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC224" t="n">
         <v>33621</v>
       </c>
-      <c r="AC224" t="n">
+      <c r="AD224" t="n">
         <v>135</v>
       </c>
     </row>
@@ -21109,9 +21784,12 @@
         <v>87</v>
       </c>
       <c r="AB225" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC225" t="n">
         <v>30133</v>
       </c>
-      <c r="AC225" t="n">
+      <c r="AD225" t="n">
         <v>506</v>
       </c>
     </row>
@@ -21208,9 +21886,12 @@
         <v>102</v>
       </c>
       <c r="AB226" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC226" t="n">
         <v>33848</v>
       </c>
-      <c r="AC226" t="n">
+      <c r="AD226" t="n">
         <v>300</v>
       </c>
     </row>
@@ -21313,9 +21994,12 @@
         <v>130</v>
       </c>
       <c r="AB227" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC227" t="n">
         <v>32530</v>
       </c>
-      <c r="AC227" t="n">
+      <c r="AD227" t="n">
         <v>431</v>
       </c>
     </row>
@@ -21418,9 +22102,12 @@
         <v>96</v>
       </c>
       <c r="AB228" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC228" t="n">
         <v>31554</v>
       </c>
-      <c r="AC228" t="n">
+      <c r="AD228" t="n">
         <v>632</v>
       </c>
     </row>
@@ -21517,9 +22204,12 @@
         <v>101</v>
       </c>
       <c r="AB229" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC229" t="n">
         <v>30874</v>
       </c>
-      <c r="AC229" t="n">
+      <c r="AD229" t="n">
         <v>180</v>
       </c>
     </row>
@@ -21619,9 +22309,12 @@
         <v>125</v>
       </c>
       <c r="AB230" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC230" t="n">
         <v>33754</v>
       </c>
-      <c r="AC230" t="n">
+      <c r="AD230" t="n">
         <v>235</v>
       </c>
     </row>
@@ -21723,9 +22416,12 @@
         <v>129</v>
       </c>
       <c r="AB231" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC231" t="n">
         <v>34776</v>
       </c>
-      <c r="AC231" t="n">
+      <c r="AD231" t="n">
         <v>313</v>
       </c>
     </row>
@@ -21827,9 +22523,12 @@
         <v>113</v>
       </c>
       <c r="AB232" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC232" t="n">
         <v>32512</v>
       </c>
-      <c r="AC232" t="n">
+      <c r="AD232" t="n">
         <v>290</v>
       </c>
     </row>
@@ -21930,9 +22629,12 @@
         <v>139</v>
       </c>
       <c r="AB233" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC233" t="n">
         <v>34815</v>
       </c>
-      <c r="AC233" t="n">
+      <c r="AD233" t="n">
         <v>311</v>
       </c>
     </row>
@@ -22035,9 +22737,12 @@
         <v>92</v>
       </c>
       <c r="AB234" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC234" t="n">
         <v>33589</v>
       </c>
-      <c r="AC234" t="n">
+      <c r="AD234" t="n">
         <v>538</v>
       </c>
     </row>
@@ -22137,9 +22842,12 @@
         <v>124</v>
       </c>
       <c r="AB235" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC235" t="n">
         <v>32826</v>
       </c>
-      <c r="AC235" t="n">
+      <c r="AD235" t="n">
         <v>352</v>
       </c>
     </row>
@@ -22239,9 +22947,12 @@
         <v>128</v>
       </c>
       <c r="AB236" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC236" t="n">
         <v>34663</v>
       </c>
-      <c r="AC236" t="n">
+      <c r="AD236" t="n">
         <v>396</v>
       </c>
     </row>
@@ -22348,9 +23059,12 @@
         <v>137</v>
       </c>
       <c r="AB237" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC237" t="n">
         <v>32556</v>
       </c>
-      <c r="AC237" t="n">
+      <c r="AD237" t="n">
         <v>626</v>
       </c>
     </row>
@@ -22451,9 +23165,12 @@
         <v>144</v>
       </c>
       <c r="AB238" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC238" t="n">
         <v>34180</v>
       </c>
-      <c r="AC238" t="n">
+      <c r="AD238" t="n">
         <v>408</v>
       </c>
     </row>
@@ -22554,9 +23271,12 @@
         <v>82</v>
       </c>
       <c r="AB239" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC239" t="n">
         <v>30571</v>
       </c>
-      <c r="AC239" t="n">
+      <c r="AD239" t="n">
         <v>307</v>
       </c>
     </row>
@@ -22656,9 +23376,12 @@
         <v>160</v>
       </c>
       <c r="AB240" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC240" t="n">
         <v>34339</v>
       </c>
-      <c r="AC240" t="n">
+      <c r="AD240" t="n">
         <v>429</v>
       </c>
     </row>
@@ -22759,9 +23482,12 @@
         <v>84</v>
       </c>
       <c r="AB241" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC241" t="n">
         <v>32886</v>
       </c>
-      <c r="AC241" t="n">
+      <c r="AD241" t="n">
         <v>378</v>
       </c>
     </row>
@@ -22861,9 +23587,12 @@
         <v>149</v>
       </c>
       <c r="AB242" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC242" t="n">
         <v>34733</v>
       </c>
-      <c r="AC242" t="n">
+      <c r="AD242" t="n">
         <v>872</v>
       </c>
     </row>
@@ -22967,9 +23696,12 @@
         <v>78</v>
       </c>
       <c r="AB243" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC243" t="n">
         <v>29357</v>
       </c>
-      <c r="AC243" t="n">
+      <c r="AD243" t="n">
         <v>523</v>
       </c>
     </row>
@@ -23072,9 +23804,12 @@
         <v>100</v>
       </c>
       <c r="AB244" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC244" t="n">
         <v>30351</v>
       </c>
-      <c r="AC244" t="n">
+      <c r="AD244" t="n">
         <v>403</v>
       </c>
     </row>
@@ -23171,9 +23906,12 @@
         <v>160</v>
       </c>
       <c r="AB245" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC245" t="n">
         <v>34588</v>
       </c>
-      <c r="AC245" t="n">
+      <c r="AD245" t="n">
         <v>217</v>
       </c>
     </row>
@@ -23275,9 +24013,12 @@
         <v>109</v>
       </c>
       <c r="AB246" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC246" t="n">
         <v>30306</v>
       </c>
-      <c r="AC246" t="n">
+      <c r="AD246" t="n">
         <v>404</v>
       </c>
     </row>
@@ -23380,9 +24121,12 @@
         <v>93</v>
       </c>
       <c r="AB247" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC247" t="n">
         <v>29817</v>
       </c>
-      <c r="AC247" t="n">
+      <c r="AD247" t="n">
         <v>397</v>
       </c>
     </row>
@@ -23485,9 +24229,12 @@
         <v>119</v>
       </c>
       <c r="AB248" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC248" t="n">
         <v>31988</v>
       </c>
-      <c r="AC248" t="n">
+      <c r="AD248" t="n">
         <v>433</v>
       </c>
     </row>
@@ -23584,9 +24331,12 @@
         <v>109</v>
       </c>
       <c r="AB249" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC249" t="n">
         <v>34847</v>
       </c>
-      <c r="AC249" t="n">
+      <c r="AD249" t="n">
         <v>140</v>
       </c>
     </row>
@@ -23683,9 +24433,12 @@
         <v>156</v>
       </c>
       <c r="AB250" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC250" t="n">
         <v>32527</v>
       </c>
-      <c r="AC250" t="n">
+      <c r="AD250" t="n">
         <v>288</v>
       </c>
     </row>
@@ -23782,9 +24535,12 @@
         <v>226</v>
       </c>
       <c r="AB251" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC251" t="n">
         <v>33114</v>
       </c>
-      <c r="AC251" t="n">
+      <c r="AD251" t="n">
         <v>223</v>
       </c>
     </row>
@@ -23884,9 +24640,12 @@
         <v>77</v>
       </c>
       <c r="AB252" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC252" t="n">
         <v>33005</v>
       </c>
-      <c r="AC252" t="n">
+      <c r="AD252" t="n">
         <v>763</v>
       </c>
     </row>
@@ -23985,9 +24744,12 @@
         <v>179</v>
       </c>
       <c r="AB253" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC253" t="n">
         <v>35412</v>
       </c>
-      <c r="AC253" t="n">
+      <c r="AD253" t="n">
         <v>283</v>
       </c>
     </row>
@@ -24086,9 +24848,12 @@
         <v>126</v>
       </c>
       <c r="AB254" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC254" t="n">
         <v>32228</v>
       </c>
-      <c r="AC254" t="n">
+      <c r="AD254" t="n">
         <v>340</v>
       </c>
     </row>
@@ -24185,9 +24950,12 @@
         <v>144</v>
       </c>
       <c r="AB255" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC255" t="n">
         <v>33986</v>
       </c>
-      <c r="AC255" t="n">
+      <c r="AD255" t="n">
         <v>192</v>
       </c>
     </row>
@@ -24284,9 +25052,12 @@
         <v>106</v>
       </c>
       <c r="AB256" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC256" t="n">
         <v>34194</v>
       </c>
-      <c r="AC256" t="n">
+      <c r="AD256" t="n">
         <v>370</v>
       </c>
     </row>
@@ -24386,9 +25157,12 @@
         <v>107</v>
       </c>
       <c r="AB257" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC257" t="n">
         <v>32089</v>
       </c>
-      <c r="AC257" t="n">
+      <c r="AD257" t="n">
         <v>249</v>
       </c>
     </row>
@@ -24502,9 +25276,12 @@
         <v>137</v>
       </c>
       <c r="AB258" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC258" t="n">
         <v>34680</v>
       </c>
-      <c r="AC258" t="n">
+      <c r="AD258" t="n">
         <v>872</v>
       </c>
     </row>
@@ -24607,9 +25384,12 @@
         <v>79</v>
       </c>
       <c r="AB259" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC259" t="n">
         <v>32809</v>
       </c>
-      <c r="AC259" t="n">
+      <c r="AD259" t="n">
         <v>402</v>
       </c>
     </row>
@@ -24713,9 +25493,12 @@
         <v>96</v>
       </c>
       <c r="AB260" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC260" t="n">
         <v>31520</v>
       </c>
-      <c r="AC260" t="n">
+      <c r="AD260" t="n">
         <v>507</v>
       </c>
     </row>
@@ -24820,9 +25603,12 @@
         <v>95</v>
       </c>
       <c r="AB261" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC261" t="n">
         <v>34585</v>
       </c>
-      <c r="AC261" t="n">
+      <c r="AD261" t="n">
         <v>1162</v>
       </c>
     </row>
@@ -24919,9 +25705,12 @@
         <v>102</v>
       </c>
       <c r="AB262" t="n">
+        <v>20735</v>
+      </c>
+      <c r="AC262" t="n">
         <v>10423</v>
       </c>
-      <c r="AC262" t="n">
+      <c r="AD262" t="n">
         <v>247</v>
       </c>
     </row>
@@ -25021,9 +25810,12 @@
         <v>98</v>
       </c>
       <c r="AB263" t="n">
+        <v>55931</v>
+      </c>
+      <c r="AC263" t="n">
         <v>26861</v>
       </c>
-      <c r="AC263" t="n">
+      <c r="AD263" t="n">
         <v>334</v>
       </c>
     </row>
@@ -25128,9 +25920,12 @@
         <v>133</v>
       </c>
       <c r="AB264" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC264" t="n">
         <v>32683</v>
       </c>
-      <c r="AC264" t="n">
+      <c r="AD264" t="n">
         <v>514</v>
       </c>
     </row>
@@ -25229,9 +26024,12 @@
         <v>142</v>
       </c>
       <c r="AB265" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC265" t="n">
         <v>34720</v>
       </c>
-      <c r="AC265" t="n">
+      <c r="AD265" t="n">
         <v>265</v>
       </c>
     </row>
@@ -25334,9 +26132,12 @@
         <v>122</v>
       </c>
       <c r="AB266" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC266" t="n">
         <v>28867</v>
       </c>
-      <c r="AC266" t="n">
+      <c r="AD266" t="n">
         <v>474</v>
       </c>
     </row>
@@ -25438,9 +26239,12 @@
         <v>79</v>
       </c>
       <c r="AB267" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC267" t="n">
         <v>32186</v>
       </c>
-      <c r="AC267" t="n">
+      <c r="AD267" t="n">
         <v>520</v>
       </c>
     </row>
@@ -25542,9 +26346,12 @@
         <v>100</v>
       </c>
       <c r="AB268" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC268" t="n">
         <v>34275</v>
       </c>
-      <c r="AC268" t="n">
+      <c r="AD268" t="n">
         <v>578</v>
       </c>
     </row>
@@ -25647,9 +26454,12 @@
         <v>100</v>
       </c>
       <c r="AB269" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC269" t="n">
         <v>32211</v>
       </c>
-      <c r="AC269" t="n">
+      <c r="AD269" t="n">
         <v>498</v>
       </c>
     </row>
@@ -25753,9 +26563,12 @@
         <v>102</v>
       </c>
       <c r="AB270" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC270" t="n">
         <v>32582</v>
       </c>
-      <c r="AC270" t="n">
+      <c r="AD270" t="n">
         <v>568</v>
       </c>
     </row>
@@ -25856,9 +26669,12 @@
         <v>126</v>
       </c>
       <c r="AB271" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC271" t="n">
         <v>35676</v>
       </c>
-      <c r="AC271" t="n">
+      <c r="AD271" t="n">
         <v>382</v>
       </c>
     </row>
@@ -25955,9 +26771,12 @@
         <v>77</v>
       </c>
       <c r="AB272" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC272" t="n">
         <v>34802</v>
       </c>
-      <c r="AC272" t="n">
+      <c r="AD272" t="n">
         <v>239</v>
       </c>
     </row>
@@ -26060,9 +26879,12 @@
         <v>102</v>
       </c>
       <c r="AB273" t="n">
+        <v>70096</v>
+      </c>
+      <c r="AC273" t="n">
         <v>33622</v>
       </c>
-      <c r="AC273" t="n">
+      <c r="AD273" t="n">
         <v>358</v>
       </c>
     </row>
@@ -26162,9 +26984,12 @@
         <v>139</v>
       </c>
       <c r="AB274" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC274" t="n">
         <v>34172</v>
       </c>
-      <c r="AC274" t="n">
+      <c r="AD274" t="n">
         <v>341</v>
       </c>
     </row>
@@ -26266,9 +27091,12 @@
         <v>135</v>
       </c>
       <c r="AB275" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC275" t="n">
         <v>33932</v>
       </c>
-      <c r="AC275" t="n">
+      <c r="AD275" t="n">
         <v>368</v>
       </c>
     </row>
@@ -26369,9 +27197,12 @@
         <v>81</v>
       </c>
       <c r="AB276" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC276" t="n">
         <v>34151</v>
       </c>
-      <c r="AC276" t="n">
+      <c r="AD276" t="n">
         <v>353</v>
       </c>
     </row>
@@ -26468,9 +27299,12 @@
         <v>91</v>
       </c>
       <c r="AB277" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC277" t="n">
         <v>34194</v>
       </c>
-      <c r="AC277" t="n">
+      <c r="AD277" t="n">
         <v>329</v>
       </c>
     </row>
@@ -26567,9 +27401,12 @@
         <v>77</v>
       </c>
       <c r="AB278" t="n">
+        <v>58744</v>
+      </c>
+      <c r="AC278" t="n">
         <v>28134</v>
       </c>
-      <c r="AC278" t="n">
+      <c r="AD278" t="n">
         <v>227</v>
       </c>
     </row>
@@ -26666,9 +27503,12 @@
         <v>64</v>
       </c>
       <c r="AB279" t="n">
+        <v>68647</v>
+      </c>
+      <c r="AC279" t="n">
         <v>32974</v>
       </c>
-      <c r="AC279" t="n">
+      <c r="AD279" t="n">
         <v>205</v>
       </c>
     </row>
@@ -26765,9 +27605,12 @@
         <v>46</v>
       </c>
       <c r="AB280" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC280" t="n">
         <v>34489</v>
       </c>
-      <c r="AC280" t="n">
+      <c r="AD280" t="n">
         <v>204</v>
       </c>
     </row>
@@ -26870,9 +27713,12 @@
         <v>112</v>
       </c>
       <c r="AB281" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC281" t="n">
         <v>34475</v>
       </c>
-      <c r="AC281" t="n">
+      <c r="AD281" t="n">
         <v>645</v>
       </c>
     </row>
@@ -26971,9 +27817,12 @@
         <v>146</v>
       </c>
       <c r="AB282" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC282" t="n">
         <v>33852</v>
       </c>
-      <c r="AC282" t="n">
+      <c r="AD282" t="n">
         <v>657</v>
       </c>
     </row>
@@ -27072,9 +27921,12 @@
         <v>82</v>
       </c>
       <c r="AB283" t="n">
+        <v>33408</v>
+      </c>
+      <c r="AC283" t="n">
         <v>16523</v>
       </c>
-      <c r="AC283" t="n">
+      <c r="AD283" t="n">
         <v>258</v>
       </c>
     </row>
@@ -27177,9 +28029,12 @@
         <v>90</v>
       </c>
       <c r="AB284" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC284" t="n">
         <v>33268</v>
       </c>
-      <c r="AC284" t="n">
+      <c r="AD284" t="n">
         <v>454</v>
       </c>
     </row>
@@ -27276,9 +28131,12 @@
         <v>68</v>
       </c>
       <c r="AB285" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC285" t="n">
         <v>34353</v>
       </c>
-      <c r="AC285" t="n">
+      <c r="AD285" t="n">
         <v>246</v>
       </c>
     </row>
@@ -27375,9 +28233,12 @@
         <v>73</v>
       </c>
       <c r="AB286" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC286" t="n">
         <v>34803</v>
       </c>
-      <c r="AC286" t="n">
+      <c r="AD286" t="n">
         <v>225</v>
       </c>
     </row>
@@ -27477,9 +28338,12 @@
         <v>118</v>
       </c>
       <c r="AB287" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC287" t="n">
         <v>34242</v>
       </c>
-      <c r="AC287" t="n">
+      <c r="AD287" t="n">
         <v>275</v>
       </c>
     </row>
@@ -27576,9 +28440,12 @@
         <v>61</v>
       </c>
       <c r="AB288" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC288" t="n">
         <v>34529</v>
       </c>
-      <c r="AC288" t="n">
+      <c r="AD288" t="n">
         <v>229</v>
       </c>
     </row>
@@ -27675,9 +28542,12 @@
         <v>64</v>
       </c>
       <c r="AB289" t="n">
+        <v>64087</v>
+      </c>
+      <c r="AC289" t="n">
         <v>30898</v>
       </c>
-      <c r="AC289" t="n">
+      <c r="AD289" t="n">
         <v>198</v>
       </c>
     </row>
@@ -27780,9 +28650,12 @@
         <v>90</v>
       </c>
       <c r="AB290" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC290" t="n">
         <v>30130</v>
       </c>
-      <c r="AC290" t="n">
+      <c r="AD290" t="n">
         <v>316</v>
       </c>
     </row>
@@ -27887,9 +28760,12 @@
         <v>85</v>
       </c>
       <c r="AB291" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC291" t="n">
         <v>32059</v>
       </c>
-      <c r="AC291" t="n">
+      <c r="AD291" t="n">
         <v>393</v>
       </c>
     </row>
@@ -27986,9 +28862,12 @@
         <v>73</v>
       </c>
       <c r="AB292" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC292" t="n">
         <v>34264</v>
       </c>
-      <c r="AC292" t="n">
+      <c r="AD292" t="n">
         <v>85</v>
       </c>
     </row>
@@ -28085,9 +28964,12 @@
         <v>74</v>
       </c>
       <c r="AB293" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC293" t="n">
         <v>32519</v>
       </c>
-      <c r="AC293" t="n">
+      <c r="AD293" t="n">
         <v>226</v>
       </c>
     </row>
@@ -28193,9 +29075,12 @@
         <v>60</v>
       </c>
       <c r="AB294" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC294" t="n">
         <v>31412</v>
       </c>
-      <c r="AC294" t="n">
+      <c r="AD294" t="n">
         <v>492</v>
       </c>
     </row>
@@ -28297,9 +29182,12 @@
         <v>84</v>
       </c>
       <c r="AB295" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC295" t="n">
         <v>32090</v>
       </c>
-      <c r="AC295" t="n">
+      <c r="AD295" t="n">
         <v>331</v>
       </c>
     </row>
@@ -28400,9 +29288,12 @@
         <v>71</v>
       </c>
       <c r="AB296" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC296" t="n">
         <v>32685</v>
       </c>
-      <c r="AC296" t="n">
+      <c r="AD296" t="n">
         <v>349</v>
       </c>
     </row>
@@ -28499,9 +29390,12 @@
         <v>103</v>
       </c>
       <c r="AB297" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC297" t="n">
         <v>33017</v>
       </c>
-      <c r="AC297" t="n">
+      <c r="AD297" t="n">
         <v>331</v>
       </c>
     </row>
@@ -28598,9 +29492,12 @@
         <v>90</v>
       </c>
       <c r="AB298" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC298" t="n">
         <v>33550</v>
       </c>
-      <c r="AC298" t="n">
+      <c r="AD298" t="n">
         <v>99</v>
       </c>
     </row>
@@ -28697,9 +29594,12 @@
         <v>82</v>
       </c>
       <c r="AB299" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC299" t="n">
         <v>33884</v>
       </c>
-      <c r="AC299" t="n">
+      <c r="AD299" t="n">
         <v>116</v>
       </c>
     </row>
@@ -28804,9 +29704,12 @@
         <v>71</v>
       </c>
       <c r="AB300" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC300" t="n">
         <v>30815</v>
       </c>
-      <c r="AC300" t="n">
+      <c r="AD300" t="n">
         <v>341</v>
       </c>
     </row>
@@ -28914,14 +29817,17 @@
         <v>66</v>
       </c>
       <c r="AB301" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AC301" t="n">
         <v>31246</v>
       </c>
-      <c r="AC301" t="n">
+      <c r="AD301" t="n">
         <v>447</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC301"/>
+  <autoFilter ref="A1:AD301"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -28932,10 +29838,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
@@ -29478,32 +30384,48 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>answer_tokens_in</t>
+          <t>retrieved_context_characters</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>26281.19</v>
+        <v>72000</v>
       </c>
       <c r="C39" t="n">
-        <v>30165.13</v>
+        <v>72000</v>
       </c>
       <c r="D39" t="n">
-        <v>32440.12</v>
+        <v>70676.48</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>answer_tokens_in</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>26281.19</v>
+      </c>
+      <c r="C40" t="n">
+        <v>30165.13</v>
+      </c>
+      <c r="D40" t="n">
+        <v>32440.12</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>answer_tokens_out</t>
         </is>
       </c>
-      <c r="B40" t="n">
+      <c r="B41" t="n">
         <v>317.86</v>
       </c>
-      <c r="C40" t="n">
+      <c r="C41" t="n">
         <v>427.55</v>
       </c>
-      <c r="D40" t="n">
+      <c r="D41" t="n">
         <v>373.96</v>
       </c>
     </row>
@@ -29766,7 +30688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -30379,17 +31301,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>answer_tokens_in</t>
+          <t>retrieved_context_characters</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Input tokens of the answer model call.</t>
+          <t>Characters of the retrieved context given to the answer model. At most character_limit.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>characters</t>
         </is>
       </c>
     </row>
@@ -30401,12 +31323,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>answer_tokens_out</t>
+          <t>answer_tokens_in</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Output tokens of the answer model call.</t>
+          <t>Input tokens of the answer model call.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -30418,22 +31340,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>run data</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>character_limit</t>
+          <t>answer_tokens_out</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Maximum characters of retrieved text given to the answer model per question.</t>
+          <t>Output tokens of the answer model call.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>characters</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
@@ -30445,15 +31367,19 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>answer_model</t>
+          <t>character_limit</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Language model of the answers and of the artefact's interpreter.</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
+          <t>Maximum characters of retrieved text given to the answer model per question.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>characters</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -30463,12 +31389,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>judge_model</t>
+          <t>answer_model</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Language model that RAGAS uses as judge.</t>
+          <t>Language model of the answers and of the artefact's interpreter.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -30481,12 +31407,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>embedding_model</t>
+          <t>judge_model</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Embedding model of the query embeddings and of the RAGAS scores that use embeddings.</t>
+          <t>Language model that RAGAS uses as judge.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -30499,19 +31425,15 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>run_seconds</t>
+          <t>embedding_model</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Time of the run over the 100 questions, without failed tries of model calls.</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
+          <t>Embedding model of the query embeddings and of the RAGAS scores that use embeddings.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -30521,17 +31443,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>judge_tokens_in</t>
+          <t>run_seconds</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Input tokens of all RAGAS judge calls.</t>
+          <t>Time of the run over the 100 questions, without failed tries of model calls.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
@@ -30543,12 +31465,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>judge_tokens_out</t>
+          <t>judge_tokens_in</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Output tokens of all RAGAS judge calls.</t>
+          <t>Input tokens of all RAGAS judge calls.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -30565,12 +31487,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>judge_embedding_tokens</t>
+          <t>judge_tokens_out</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Tokens embedded by RAGAS.</t>
+          <t>Output tokens of all RAGAS judge calls.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -30587,17 +31509,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>judging_seconds</t>
+          <t>judge_embedding_tokens</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Time of the RAGAS evaluation over the 100 questions.</t>
+          <t>Tokens embedded by RAGAS.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>seconds</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
@@ -30609,30 +31531,34 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>mean of</t>
+          <t>judging_seconds</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mean over the arm's 100 questions of the field of results named in the row.</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
+          <t>Time of the RAGAS evaluation over the 100 questions.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>arm construction</t>
+          <t>run data</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>mean of</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Index type.</t>
+          <t>Mean over the arm's 100 questions of the field of results named in the row.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -30645,12 +31571,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>index</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Unit stored in the index.</t>
+          <t>Index type.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -30663,19 +31589,15 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>units in the index</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Units in the index.</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
+          <t>Unit stored in the index.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -30685,17 +31607,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>build time, seconds</t>
+          <t>units in the index</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Time to build the index. Artefact: sum of the times of the build steps.</t>
+          <t>Units in the index.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>seconds</t>
+          <t>count</t>
         </is>
       </c>
     </row>
@@ -30707,17 +31629,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
+          <t>build time, seconds</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Texts embedded for the index.</t>
+          <t>Time to build the index. Artefact: sum of the times of the build steps.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
@@ -30729,17 +31651,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, tokens</t>
+          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Tokens embedded for the index.</t>
+          <t>Texts embedded for the index.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>count</t>
         </is>
       </c>
     </row>
@@ -30751,17 +31673,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, seconds</t>
+          <t>llama-nemotron-embed-1b-v2, tokens</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Embedding time for the index.</t>
+          <t>Tokens embedded for the index.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>seconds</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
@@ -30773,17 +31695,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, calls</t>
+          <t>llama-nemotron-embed-1b-v2, seconds</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Calls to claude-haiku-4-5 for the index.</t>
+          <t>Embedding time for the index.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
@@ -30795,17 +31717,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, tokens in</t>
+          <t>claude-haiku-4-5, calls</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Input tokens of those calls.</t>
+          <t>Calls to claude-haiku-4-5 for the index.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>count</t>
         </is>
       </c>
     </row>
@@ -30817,12 +31739,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, tokens out</t>
+          <t>claude-haiku-4-5, tokens in</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Output tokens of those calls.</t>
+          <t>Input tokens of those calls.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -30839,17 +31761,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, seconds</t>
+          <t>claude-haiku-4-5, tokens out</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Time of those calls: the time of the pass that made them, multiplied by their share of the pass's call time.</t>
+          <t>Output tokens of those calls.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>seconds</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
@@ -30861,17 +31783,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>claude-opus-5, calls</t>
+          <t>claude-haiku-4-5, seconds</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Calls to claude-opus-5 for the index.</t>
+          <t>Time of those calls: the time of the pass that made them, multiplied by their share of the pass's call time.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
@@ -30883,17 +31805,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>claude-opus-5, tokens in</t>
+          <t>claude-opus-5, calls</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Input tokens of those calls.</t>
+          <t>Calls to claude-opus-5 for the index.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>count</t>
         </is>
       </c>
     </row>
@@ -30905,12 +31827,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>claude-opus-5, tokens out</t>
+          <t>claude-opus-5, tokens in</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Output tokens of those calls.</t>
+          <t>Input tokens of those calls.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -30927,17 +31849,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>claude-opus-5, seconds</t>
+          <t>claude-opus-5, tokens out</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Time of those calls.</t>
+          <t>Output tokens of those calls.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>seconds</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
@@ -30949,22 +31871,44 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>claude-opus-5, seconds</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Time of those calls.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>arm construction</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>gte-reranker-modernbert-base, seconds</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>Encoding time of gte-reranker-modernbert-base for the index.</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>seconds</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D56"/>
+  <autoFilter ref="A1:D57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
export: the split run's time is the added time of all the things in it, as for the other arms; its judging the same way
</commit_message>
<xml_diff>
--- a/finished_data/grag-data.xlsx
+++ b/finished_data/grag-data.xlsx
@@ -29933,7 +29933,7 @@
         <v>901.5495188999921</v>
       </c>
       <c r="D10" t="n">
-        <v>190.403121</v>
+        <v>5986.179287903404</v>
       </c>
     </row>
     <row r="11">
@@ -29997,7 +29997,7 @@
         <v>4232.659700700082</v>
       </c>
       <c r="D14" t="n">
-        <v>561.9581460000001</v>
+        <v>2488.393881</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
export: every arm's run time and judging time is its questions' times added, never the run's clock; the workbook made again
</commit_message>
<xml_diff>
--- a/finished_data/grag-data.xlsx
+++ b/finished_data/grag-data.xlsx
@@ -29980,13 +29980,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>680.8228764000814</v>
+        <v>676.77251870092</v>
       </c>
       <c r="C10" t="n">
-        <v>901.5495188999921</v>
+        <v>866.7278056973591</v>
       </c>
       <c r="D10" t="n">
-        <v>164.985167200095</v>
+        <v>4724.015682603465</v>
       </c>
     </row>
     <row r="11">
@@ -30044,13 +30044,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4471.126690400066</v>
+        <v>4129.70354</v>
       </c>
       <c r="C14" t="n">
-        <v>4232.659700700082</v>
+        <v>3769.242378</v>
       </c>
       <c r="D14" t="n">
-        <v>524.1787285000319</v>
+        <v>3631.450524</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
the vector and lucene runs on the 715 answerable questions, the vector run's 612 zero answer-call token counts corrected; the lane's API-key fallback on HTTP 429, the 128000 output cap and the 1h cache; the GPU embedding-time corrections of the final runs; the non-LLM record-content tools; the six files over 100 MB kept out (copied between the machines)
</commit_message>
<xml_diff>
--- a/finished_data/grag-data.xlsx
+++ b/finished_data/grag-data.xlsx
@@ -11324,13 +11324,13 @@
         <v>0.3889033002778888</v>
       </c>
       <c r="Z102" t="n">
-        <v>0.9214409999549389</v>
+        <v>0.0271084998967126</v>
       </c>
       <c r="AA102" t="n">
         <v>16.52928970009089</v>
       </c>
       <c r="AB102" t="n">
-        <v>17.85192599985749</v>
+        <v>16.95759349979926</v>
       </c>
       <c r="AE102" t="n">
         <v>24</v>
@@ -11438,13 +11438,13 @@
         <v>0.04714470030739903</v>
       </c>
       <c r="Z103" t="n">
-        <v>0.3443478997796774</v>
+        <v>0.02455699967686087</v>
       </c>
       <c r="AA103" t="n">
         <v>5.606997199822217</v>
       </c>
       <c r="AB103" t="n">
-        <v>6.01016389997676</v>
+        <v>5.690372999873944</v>
       </c>
       <c r="AE103" t="n">
         <v>22</v>
@@ -11547,13 +11547,13 @@
         <v>0.1357296998612583</v>
       </c>
       <c r="Z104" t="n">
-        <v>0.729903600178659</v>
+        <v>0.02364920009858906</v>
       </c>
       <c r="AA104" t="n">
         <v>5.456526999827474</v>
       </c>
       <c r="AB104" t="n">
-        <v>6.336764900013804</v>
+        <v>5.630510499933735</v>
       </c>
       <c r="AE104" t="n">
         <v>23</v>
@@ -11657,13 +11657,13 @@
         <v>0.08503719978034496</v>
       </c>
       <c r="Z105" t="n">
-        <v>0.9181691003032029</v>
+        <v>0.02731840021442622</v>
       </c>
       <c r="AA105" t="n">
         <v>6.329620399978012</v>
       </c>
       <c r="AB105" t="n">
-        <v>7.342884299810976</v>
+        <v>6.452033599722199</v>
       </c>
       <c r="AE105" t="n">
         <v>26</v>
@@ -11768,13 +11768,13 @@
         <v>0.08582720020785928</v>
       </c>
       <c r="Z106" t="n">
-        <v>0.7646865998394787</v>
+        <v>0.02404499996919185</v>
       </c>
       <c r="AA106" t="n">
         <v>7.172951499931514</v>
       </c>
       <c r="AB106" t="n">
-        <v>8.031202499754727</v>
+        <v>7.29056089988444</v>
       </c>
       <c r="AE106" t="n">
         <v>22</v>
@@ -11879,13 +11879,13 @@
         <v>0.06248300010338426</v>
       </c>
       <c r="Z107" t="n">
-        <v>0.3592862002551556</v>
+        <v>0.026266900007613</v>
       </c>
       <c r="AA107" t="n">
         <v>6.758090400137007</v>
       </c>
       <c r="AB107" t="n">
-        <v>7.188027199823409</v>
+        <v>6.855007899575867</v>
       </c>
       <c r="AE107" t="n">
         <v>24</v>
@@ -11991,13 +11991,13 @@
         <v>0.06239399965852499</v>
       </c>
       <c r="Z108" t="n">
-        <v>0.4114784998819232</v>
+        <v>0.02512810006737709</v>
       </c>
       <c r="AA108" t="n">
         <v>6.966193200089037</v>
       </c>
       <c r="AB108" t="n">
-        <v>7.457051699981093</v>
+        <v>7.070701300166547</v>
       </c>
       <c r="AE108" t="n">
         <v>31</v>
@@ -12101,13 +12101,13 @@
         <v>0.07753110025078058</v>
       </c>
       <c r="Z109" t="n">
-        <v>0.6567787998355925</v>
+        <v>0.02435720001813024</v>
       </c>
       <c r="AA109" t="n">
         <v>6.015834799967706</v>
       </c>
       <c r="AB109" t="n">
-        <v>6.761922199744731</v>
+        <v>6.129500599927269</v>
       </c>
       <c r="AE109" t="n">
         <v>22</v>
@@ -12210,13 +12210,13 @@
         <v>0.08911420032382011</v>
       </c>
       <c r="Z110" t="n">
-        <v>0.5946062998846173</v>
+        <v>0.02543459995649755</v>
       </c>
       <c r="AA110" t="n">
         <v>6.708198999986053</v>
       </c>
       <c r="AB110" t="n">
-        <v>7.401231999974698</v>
+        <v>6.832060300046578</v>
       </c>
       <c r="AE110" t="n">
         <v>19</v>
@@ -12319,13 +12319,13 @@
         <v>0.04072029981762171</v>
       </c>
       <c r="Z111" t="n">
-        <v>0.3738732999190688</v>
+        <v>0.03950489999260753</v>
       </c>
       <c r="AA111" t="n">
         <v>5.135089999996126</v>
       </c>
       <c r="AB111" t="n">
-        <v>5.562333399895579</v>
+        <v>5.227964999969117</v>
       </c>
       <c r="AE111" t="n">
         <v>19</v>
@@ -12433,13 +12433,13 @@
         <v>0.08891469985246658</v>
       </c>
       <c r="Z112" t="n">
-        <v>0.6605184003710747</v>
+        <v>0.02765990037005395</v>
       </c>
       <c r="AA112" t="n">
         <v>7.406391200143844</v>
       </c>
       <c r="AB112" t="n">
-        <v>8.169692699797451</v>
+        <v>7.536834199796431</v>
       </c>
       <c r="AE112" t="n">
         <v>30</v>
@@ -12550,13 +12550,13 @@
         <v>0.04372119996696711</v>
       </c>
       <c r="Z113" t="n">
-        <v>0.3317234995774925</v>
+        <v>0.02538309991359711</v>
       </c>
       <c r="AA113" t="n">
         <v>8.008816900197417</v>
       </c>
       <c r="AB113" t="n">
-        <v>8.399264399893582</v>
+        <v>8.092924000229686</v>
       </c>
       <c r="AE113" t="n">
         <v>17</v>
@@ -12659,13 +12659,13 @@
         <v>0.09325960045680404</v>
       </c>
       <c r="Z114" t="n">
-        <v>0.8346556997857988</v>
+        <v>0.02576430002227426</v>
       </c>
       <c r="AA114" t="n">
         <v>9.131965199951082</v>
       </c>
       <c r="AB114" t="n">
-        <v>10.07566240010783</v>
+        <v>9.266771000344306</v>
       </c>
       <c r="AE114" t="n">
         <v>19</v>
@@ -12772,13 +12772,13 @@
         <v>0.08019069954752922</v>
       </c>
       <c r="Z115" t="n">
-        <v>0.557734000030905</v>
+        <v>0.027313900180161</v>
       </c>
       <c r="AA115" t="n">
         <v>7.89159579994157</v>
       </c>
       <c r="AB115" t="n">
-        <v>8.542528600431979</v>
+        <v>8.012108500581235</v>
       </c>
       <c r="AE115" t="n">
         <v>17</v>
@@ -12891,13 +12891,13 @@
         <v>0.04180529993027449</v>
       </c>
       <c r="Z116" t="n">
-        <v>0.3319306001067162</v>
+        <v>0.02541860030032694</v>
       </c>
       <c r="AA116" t="n">
         <v>11.60224219970405</v>
       </c>
       <c r="AB116" t="n">
-        <v>11.98589760018513</v>
+        <v>11.67938560037874</v>
       </c>
       <c r="AE116" t="n">
         <v>21</v>
@@ -13016,13 +13016,13 @@
         <v>0.08720469987019897</v>
       </c>
       <c r="Z117" t="n">
-        <v>0.5053053996525705</v>
+        <v>0.02454229991417378</v>
       </c>
       <c r="AA117" t="n">
         <v>9.404897400178015</v>
       </c>
       <c r="AB117" t="n">
-        <v>10.00826649973169</v>
+        <v>9.527503399993293</v>
       </c>
       <c r="AE117" t="n">
         <v>22</v>
@@ -13125,13 +13125,13 @@
         <v>0.0429038000293076</v>
       </c>
       <c r="Z118" t="n">
-        <v>0.3580680000595748</v>
+        <v>0.02486789983231574</v>
       </c>
       <c r="AA118" t="n">
         <v>5.932723300065845</v>
       </c>
       <c r="AB118" t="n">
-        <v>6.346031900029629</v>
+        <v>6.01283179980237</v>
       </c>
       <c r="AE118" t="n">
         <v>18</v>
@@ -13239,13 +13239,13 @@
         <v>0.04241370037198067</v>
       </c>
       <c r="Z119" t="n">
-        <v>0.4310320997610688</v>
+        <v>0.02833930018823594</v>
       </c>
       <c r="AA119" t="n">
         <v>8.369928599800915</v>
       </c>
       <c r="AB119" t="n">
-        <v>8.861133699771017</v>
+        <v>8.458440900198184</v>
       </c>
       <c r="AE119" t="n">
         <v>24</v>
@@ -13349,13 +13349,13 @@
         <v>0.07650560047477484</v>
       </c>
       <c r="Z120" t="n">
-        <v>0.8498774999752641</v>
+        <v>0.02806229959242046</v>
       </c>
       <c r="AA120" t="n">
         <v>6.389379599597305</v>
       </c>
       <c r="AB120" t="n">
-        <v>7.333555500023067</v>
+        <v>6.511740299640223</v>
       </c>
       <c r="AE120" t="n">
         <v>22</v>
@@ -13461,13 +13461,13 @@
         <v>0.07299809996038675</v>
       </c>
       <c r="Z121" t="n">
-        <v>0.6791760995984077</v>
+        <v>0.02622019988484681</v>
       </c>
       <c r="AA121" t="n">
         <v>5.466611600015312</v>
       </c>
       <c r="AB121" t="n">
-        <v>6.233839699998498</v>
+        <v>5.580883800284937</v>
       </c>
       <c r="AE121" t="n">
         <v>17</v>
@@ -13578,13 +13578,13 @@
         <v>0.09347649943083525</v>
       </c>
       <c r="Z122" t="n">
-        <v>0.7404432999901474</v>
+        <v>0.02429980027955025</v>
       </c>
       <c r="AA122" t="n">
         <v>6.263532899785787</v>
       </c>
       <c r="AB122" t="n">
-        <v>7.108770600054413</v>
+        <v>6.392627100343816</v>
       </c>
       <c r="AE122" t="n">
         <v>21</v>
@@ -13691,13 +13691,13 @@
         <v>0.06649639969691634</v>
       </c>
       <c r="Z123" t="n">
-        <v>0.4012907003052533</v>
+        <v>0.02572340006008744</v>
       </c>
       <c r="AA123" t="n">
         <v>6.725098800379783</v>
       </c>
       <c r="AB123" t="n">
-        <v>7.207069899886847</v>
+        <v>6.831502599641681</v>
       </c>
       <c r="AE123" t="n">
         <v>15</v>
@@ -13800,13 +13800,13 @@
         <v>0.09184639994055033</v>
       </c>
       <c r="Z124" t="n">
-        <v>1.00264810025692</v>
+        <v>0.02423720003571361</v>
       </c>
       <c r="AA124" t="n">
         <v>6.781365499831736</v>
       </c>
       <c r="AB124" t="n">
-        <v>7.886540099978447</v>
+        <v>6.908129199757241</v>
       </c>
       <c r="AE124" t="n">
         <v>18</v>
@@ -13924,13 +13924,13 @@
         <v>0.07318189973011613</v>
       </c>
       <c r="Z125" t="n">
-        <v>0.3773197997361422</v>
+        <v>0.02592490008100867</v>
       </c>
       <c r="AA125" t="n">
         <v>7.840833799913526</v>
       </c>
       <c r="AB125" t="n">
-        <v>8.304938999935985</v>
+        <v>7.953544100280851</v>
       </c>
       <c r="AE125" t="n">
         <v>14</v>
@@ -14033,13 +14033,13 @@
         <v>0.08646270027384162</v>
       </c>
       <c r="Z126" t="n">
-        <v>0.7950881998986006</v>
+        <v>0.02498670015484095</v>
       </c>
       <c r="AA126" t="n">
         <v>5.60296790022403</v>
       </c>
       <c r="AB126" t="n">
-        <v>6.499407399911433</v>
+        <v>5.729305900167674</v>
       </c>
       <c r="AE126" t="n">
         <v>20</v>
@@ -14147,13 +14147,13 @@
         <v>0.06495890021324158</v>
       </c>
       <c r="Z127" t="n">
-        <v>0.4667845000512898</v>
+        <v>0.02470039983745664</v>
       </c>
       <c r="AA127" t="n">
         <v>6.389201899990439</v>
       </c>
       <c r="AB127" t="n">
-        <v>6.937422899994999</v>
+        <v>6.495338799781166</v>
       </c>
       <c r="AE127" t="n">
         <v>26</v>
@@ -14267,13 +14267,13 @@
         <v>0.1033908999525011</v>
       </c>
       <c r="Z128" t="n">
-        <v>0.8924843999557197</v>
+        <v>0.02442700043320656</v>
       </c>
       <c r="AA128" t="n">
         <v>10.44192560017109</v>
       </c>
       <c r="AB128" t="n">
-        <v>11.45707720005885</v>
+        <v>10.58901980053633</v>
       </c>
       <c r="AE128" t="n">
         <v>15</v>
@@ -14376,13 +14376,13 @@
         <v>0.04269429994747043</v>
       </c>
       <c r="Z129" t="n">
-        <v>0.365470299962908</v>
+        <v>0.0243378997547552</v>
       </c>
       <c r="AA129" t="n">
         <v>6.741150099784136</v>
       </c>
       <c r="AB129" t="n">
-        <v>7.169243900105357</v>
+        <v>6.828111499897204</v>
       </c>
       <c r="AE129" t="n">
         <v>18</v>
@@ -14488,13 +14488,13 @@
         <v>0.05580820050090551</v>
       </c>
       <c r="Z130" t="n">
-        <v>0.3860829998739064</v>
+        <v>0.02461409976240247</v>
       </c>
       <c r="AA130" t="n">
         <v>5.314628500025719</v>
       </c>
       <c r="AB130" t="n">
-        <v>5.776750100310892</v>
+        <v>5.415281200199388</v>
       </c>
       <c r="AE130" t="n">
         <v>19</v>
@@ -14602,13 +14602,13 @@
         <v>0.07919389987364411</v>
       </c>
       <c r="Z131" t="n">
-        <v>0.5632140999659896</v>
+        <v>0.02465529961045831</v>
       </c>
       <c r="AA131" t="n">
         <v>8.738546399865299</v>
       </c>
       <c r="AB131" t="n">
-        <v>9.398459400050342</v>
+        <v>8.859900599694811</v>
       </c>
       <c r="AE131" t="n">
         <v>32</v>
@@ -14721,13 +14721,13 @@
         <v>0.07698029978200793</v>
       </c>
       <c r="Z132" t="n">
-        <v>0.7549217003397644</v>
+        <v>0.02428080013487488</v>
       </c>
       <c r="AA132" t="n">
         <v>13.52730339998379</v>
       </c>
       <c r="AB132" t="n">
-        <v>14.37007350008935</v>
+        <v>13.63943259988446</v>
       </c>
       <c r="AE132" t="n">
         <v>21</v>
@@ -14830,13 +14830,13 @@
         <v>0.04345040023326874</v>
       </c>
       <c r="Z133" t="n">
-        <v>0.3654314996674657</v>
+        <v>0.02490769955329597</v>
       </c>
       <c r="AA133" t="n">
         <v>6.287248400039971</v>
       </c>
       <c r="AB133" t="n">
-        <v>6.705374599900097</v>
+        <v>6.364850799785927</v>
       </c>
       <c r="AE133" t="n">
         <v>24</v>
@@ -14950,13 +14950,13 @@
         <v>0.04681540001183748</v>
       </c>
       <c r="Z134" t="n">
-        <v>0.3232141998596489</v>
+        <v>0.0241355998441577</v>
       </c>
       <c r="AA134" t="n">
         <v>10.48795009963214</v>
       </c>
       <c r="AB134" t="n">
-        <v>10.8686696998775</v>
+        <v>10.56959109986201</v>
       </c>
       <c r="AE134" t="n">
         <v>20</v>
@@ -15064,13 +15064,13 @@
         <v>0.1071603996679187</v>
       </c>
       <c r="Z135" t="n">
-        <v>0.6866982001811266</v>
+        <v>0.02550109999720007</v>
       </c>
       <c r="AA135" t="n">
         <v>9.254570399876684</v>
       </c>
       <c r="AB135" t="n">
-        <v>10.0625994997099</v>
+        <v>9.401402399525978</v>
       </c>
       <c r="AE135" t="n">
         <v>24</v>
@@ -15176,13 +15176,13 @@
         <v>0.04563670000061393</v>
       </c>
       <c r="Z136" t="n">
-        <v>0.5584933999925852</v>
+        <v>0.02423230034764856</v>
       </c>
       <c r="AA136" t="n">
         <v>6.31365770008415</v>
       </c>
       <c r="AB136" t="n">
-        <v>6.944190099835396</v>
+        <v>6.409929000190459</v>
       </c>
       <c r="AE136" t="n">
         <v>31</v>
@@ -15293,13 +15293,13 @@
         <v>0.04530239989981055</v>
       </c>
       <c r="Z137" t="n">
-        <v>0.3548513003624976</v>
+        <v>0.02729220013134181</v>
       </c>
       <c r="AA137" t="n">
         <v>11.74438040005043</v>
       </c>
       <c r="AB137" t="n">
-        <v>12.15696399984881</v>
+        <v>11.82940489961766</v>
       </c>
       <c r="AE137" t="n">
         <v>15</v>
@@ -15409,13 +15409,13 @@
         <v>0.1050309003330767</v>
       </c>
       <c r="Z138" t="n">
-        <v>0.9547542999498546</v>
+        <v>0.02906869992148131</v>
       </c>
       <c r="AA138" t="n">
         <v>11.70380500005558</v>
       </c>
       <c r="AB138" t="n">
-        <v>12.77627929998562</v>
+        <v>11.85059369995724</v>
       </c>
       <c r="AE138" t="n">
         <v>29</v>
@@ -15524,13 +15524,13 @@
         <v>0.07875860016793013</v>
       </c>
       <c r="Z139" t="n">
-        <v>0.3866155999712646</v>
+        <v>0.02481170010287315</v>
       </c>
       <c r="AA139" t="n">
         <v>8.70636499999091</v>
       </c>
       <c r="AB139" t="n">
-        <v>9.189092500135303</v>
+        <v>8.827288600266911</v>
       </c>
       <c r="AE139" t="n">
         <v>16</v>
@@ -15659,13 +15659,13 @@
         <v>0.08206159994006157</v>
       </c>
       <c r="Z140" t="n">
-        <v>0.4288412001915276</v>
+        <v>0.02455630025360733</v>
       </c>
       <c r="AA140" t="n">
         <v>17.00757210003212</v>
       </c>
       <c r="AB140" t="n">
-        <v>17.54358270019293</v>
+        <v>17.13929780025501</v>
       </c>
       <c r="AE140" t="n">
         <v>29</v>
@@ -15775,13 +15775,13 @@
         <v>0.04396599996834993</v>
       </c>
       <c r="Z141" t="n">
-        <v>0.3789512002840638</v>
+        <v>0.02326780033763498</v>
       </c>
       <c r="AA141" t="n">
         <v>7.570197599940002</v>
       </c>
       <c r="AB141" t="n">
-        <v>8.004983599763364</v>
+        <v>7.649300199816935</v>
       </c>
       <c r="AE141" t="n">
         <v>20</v>
@@ -15887,13 +15887,13 @@
         <v>0.1001362004317343</v>
       </c>
       <c r="Z142" t="n">
-        <v>0.7601463003084064</v>
+        <v>0.03001910040620714</v>
       </c>
       <c r="AA142" t="n">
         <v>6.208929700311273</v>
       </c>
       <c r="AB142" t="n">
-        <v>7.081742399837822</v>
+        <v>6.351615199935623</v>
       </c>
       <c r="AE142" t="n">
         <v>34</v>
@@ -16000,13 +16000,13 @@
         <v>0.08490340039134026</v>
       </c>
       <c r="Z143" t="n">
-        <v>0.5049074999988079</v>
+        <v>0.02371440001297742</v>
       </c>
       <c r="AA143" t="n">
         <v>7.208485900424421</v>
       </c>
       <c r="AB143" t="n">
-        <v>7.812094400171191</v>
+        <v>7.33090130018536</v>
       </c>
       <c r="AE143" t="n">
         <v>17</v>
@@ -16121,13 +16121,13 @@
         <v>0.07539249956607819</v>
       </c>
       <c r="Z144" t="n">
-        <v>0.5833340999670327</v>
+        <v>0.02661810000427067</v>
       </c>
       <c r="AA144" t="n">
         <v>9.306583099998534</v>
       </c>
       <c r="AB144" t="n">
-        <v>9.980299999937415</v>
+        <v>9.423583999974653</v>
       </c>
       <c r="AE144" t="n">
         <v>18</v>
@@ -16230,13 +16230,13 @@
         <v>0.04052079981192946</v>
       </c>
       <c r="Z145" t="n">
-        <v>0.3389146998524666</v>
+        <v>0.03307009988930076</v>
       </c>
       <c r="AA145" t="n">
         <v>6.190883400384337</v>
       </c>
       <c r="AB145" t="n">
-        <v>6.579659100156277</v>
+        <v>6.273814500193112</v>
       </c>
       <c r="AE145" t="n">
         <v>24</v>
@@ -16345,13 +16345,13 @@
         <v>0.04704550048336387</v>
       </c>
       <c r="Z146" t="n">
-        <v>0.3334511998109519</v>
+        <v>0.02440350002143532</v>
       </c>
       <c r="AA146" t="n">
         <v>8.29808699991554</v>
       </c>
       <c r="AB146" t="n">
-        <v>8.729518999811262</v>
+        <v>8.420471300021745</v>
       </c>
       <c r="AE146" t="n">
         <v>21</v>
@@ -16467,13 +16467,13 @@
         <v>0.1014445996843278</v>
       </c>
       <c r="Z147" t="n">
-        <v>1.002618300262839</v>
+        <v>0.02438150008674711</v>
       </c>
       <c r="AA147" t="n">
         <v>11.44008539989591</v>
       </c>
       <c r="AB147" t="n">
-        <v>12.56171789998189</v>
+        <v>11.58348109980579</v>
       </c>
       <c r="AE147" t="n">
         <v>18</v>
@@ -16584,13 +16584,13 @@
         <v>0.05470880027860403</v>
       </c>
       <c r="Z148" t="n">
-        <v>0.4361998001113534</v>
+        <v>0.02563190017826855</v>
       </c>
       <c r="AA148" t="n">
         <v>7.603669700212777</v>
       </c>
       <c r="AB148" t="n">
-        <v>8.103575900197029</v>
+        <v>7.693008000263944</v>
       </c>
       <c r="AE148" t="n">
         <v>28</v>
@@ -16693,13 +16693,13 @@
         <v>0.04100089985877275</v>
       </c>
       <c r="Z149" t="n">
-        <v>0.3067378997802734</v>
+        <v>0.0261323997983709</v>
       </c>
       <c r="AA149" t="n">
         <v>6.365565000101924</v>
       </c>
       <c r="AB149" t="n">
-        <v>6.743289600126445</v>
+        <v>6.462684100144543</v>
       </c>
       <c r="AE149" t="n">
         <v>20</v>
@@ -16806,13 +16806,13 @@
         <v>0.08376910025253892</v>
       </c>
       <c r="Z150" t="n">
-        <v>0.9386171996593475</v>
+        <v>0.03440010000485927</v>
       </c>
       <c r="AA150" t="n">
         <v>6.270653800107539</v>
       </c>
       <c r="AB150" t="n">
-        <v>7.305550899822265</v>
+        <v>6.401333800167777</v>
       </c>
       <c r="AE150" t="n">
         <v>33</v>
@@ -16919,13 +16919,13 @@
         <v>0.04137920029461384</v>
       </c>
       <c r="Z151" t="n">
-        <v>0.450203400105238</v>
+        <v>0.02820439974311739</v>
       </c>
       <c r="AA151" t="n">
         <v>9.737822600174695</v>
       </c>
       <c r="AB151" t="n">
-        <v>10.24967409996316</v>
+        <v>9.827675099601038</v>
       </c>
       <c r="AE151" t="n">
         <v>40</v>
@@ -17034,13 +17034,13 @@
         <v>0.04346970003098249</v>
       </c>
       <c r="Z152" t="n">
-        <v>0.3024568003602326</v>
+        <v>0.02340180007740855</v>
       </c>
       <c r="AA152" t="n">
         <v>6.948610700201243</v>
       </c>
       <c r="AB152" t="n">
-        <v>7.308513899799436</v>
+        <v>7.029458899516612</v>
       </c>
       <c r="AE152" t="n">
         <v>15</v>
@@ -17146,13 +17146,13 @@
         <v>0.04337779991328716</v>
       </c>
       <c r="Z153" t="n">
-        <v>0.4876724001951516</v>
+        <v>0.0280579001409933</v>
       </c>
       <c r="AA153" t="n">
         <v>5.733496200293303</v>
       </c>
       <c r="AB153" t="n">
-        <v>6.279093199875206</v>
+        <v>5.819478699821047</v>
       </c>
       <c r="AE153" t="n">
         <v>41</v>
@@ -17261,13 +17261,13 @@
         <v>0.097008700016886</v>
       </c>
       <c r="Z154" t="n">
-        <v>1.021101000253111</v>
+        <v>0.02696420007850975</v>
       </c>
       <c r="AA154" t="n">
         <v>10.02628979971632</v>
       </c>
       <c r="AB154" t="n">
-        <v>11.15777939977124</v>
+        <v>10.16364259959664</v>
       </c>
       <c r="AE154" t="n">
         <v>28</v>
@@ -17378,13 +17378,13 @@
         <v>0.04633969999849796</v>
       </c>
       <c r="Z155" t="n">
-        <v>0.3222313998267055</v>
+        <v>0.02453870000317693</v>
       </c>
       <c r="AA155" t="n">
         <v>12.94961650017649</v>
       </c>
       <c r="AB155" t="n">
-        <v>13.33220330020413</v>
+        <v>13.0345106003806</v>
       </c>
       <c r="AE155" t="n">
         <v>21</v>
@@ -17487,13 +17487,13 @@
         <v>0.0412304000928998</v>
       </c>
       <c r="Z156" t="n">
-        <v>0.3077903999947011</v>
+        <v>0.02437229990027845</v>
       </c>
       <c r="AA156" t="n">
         <v>5.263045300263911</v>
       </c>
       <c r="AB156" t="n">
-        <v>5.625599899794906</v>
+        <v>5.342181799700484</v>
       </c>
       <c r="AE156" t="n">
         <v>19</v>
@@ -17603,13 +17603,13 @@
         <v>0.09771199990063906</v>
       </c>
       <c r="Z157" t="n">
-        <v>0.808984000235796</v>
+        <v>0.02493940014392138</v>
       </c>
       <c r="AA157" t="n">
         <v>9.721023600082844</v>
       </c>
       <c r="AB157" t="n">
-        <v>10.64241519989446</v>
+        <v>9.858370599802583</v>
       </c>
       <c r="AE157" t="n">
         <v>17</v>
@@ -17714,13 +17714,13 @@
         <v>0.04290100000798702</v>
       </c>
       <c r="Z158" t="n">
-        <v>0.4244221998378634</v>
+        <v>0.02368209965061396</v>
       </c>
       <c r="AA158" t="n">
         <v>6.405743499752134</v>
       </c>
       <c r="AB158" t="n">
-        <v>6.881870499812067</v>
+        <v>6.481130399624817</v>
       </c>
       <c r="AE158" t="n">
         <v>25</v>
@@ -17830,13 +17830,13 @@
         <v>0.04477929975837469</v>
       </c>
       <c r="Z159" t="n">
-        <v>0.3038750998675823</v>
+        <v>0.02480849984567612</v>
       </c>
       <c r="AA159" t="n">
         <v>7.860727899707854</v>
       </c>
       <c r="AB159" t="n">
-        <v>8.225181399844587</v>
+        <v>7.946114799822681</v>
       </c>
       <c r="AE159" t="n">
         <v>19</v>
@@ -17949,13 +17949,13 @@
         <v>0.04323430033400655</v>
       </c>
       <c r="Z160" t="n">
-        <v>0.3029875997453928</v>
+        <v>0.02417709992732853</v>
       </c>
       <c r="AA160" t="n">
         <v>10.64805309986696</v>
       </c>
       <c r="AB160" t="n">
-        <v>11.00693939998746</v>
+        <v>10.72812890016939</v>
       </c>
       <c r="AE160" t="n">
         <v>19</v>
@@ -18064,13 +18064,13 @@
         <v>0.04631089977920055</v>
       </c>
       <c r="Z161" t="n">
-        <v>0.3993514999747276</v>
+        <v>0.02558119967579842</v>
       </c>
       <c r="AA161" t="n">
         <v>13.5336826001294</v>
       </c>
       <c r="AB161" t="n">
-        <v>13.98973899986595</v>
+        <v>13.61596869956702</v>
       </c>
       <c r="AE161" t="n">
         <v>27</v>
@@ -18180,13 +18180,13 @@
         <v>0.0422970000654459</v>
       </c>
       <c r="Z162" t="n">
-        <v>0.3273308998905122</v>
+        <v>0.02845770004205406</v>
       </c>
       <c r="AA162" t="n">
         <v>9.263863299973309</v>
       </c>
       <c r="AB162" t="n">
-        <v>9.659087100066245</v>
+        <v>9.360213900217786</v>
       </c>
       <c r="AE162" t="n">
         <v>22</v>
@@ -18296,13 +18296,13 @@
         <v>0.08071930008009076</v>
       </c>
       <c r="Z163" t="n">
-        <v>0.7720789001323283</v>
+        <v>0.02499099995475262</v>
       </c>
       <c r="AA163" t="n">
         <v>11.1861697002314</v>
       </c>
       <c r="AB163" t="n">
-        <v>12.0559939998202</v>
+        <v>11.30890609964263</v>
       </c>
       <c r="AE163" t="n">
         <v>20</v>
@@ -18414,13 +18414,13 @@
         <v>0.04344499995931983</v>
       </c>
       <c r="Z164" t="n">
-        <v>0.4065509997308254</v>
+        <v>0.02553429966792464</v>
       </c>
       <c r="AA164" t="n">
         <v>7.937917900271714</v>
       </c>
       <c r="AB164" t="n">
-        <v>8.401536600198597</v>
+        <v>8.020519900135696</v>
       </c>
       <c r="AE164" t="n">
         <v>19</v>
@@ -18526,13 +18526,13 @@
         <v>0.05691529996693134</v>
       </c>
       <c r="Z165" t="n">
-        <v>1.589000999927521</v>
+        <v>0.02359809970948845</v>
       </c>
       <c r="AA165" t="n">
         <v>7.781131299678236</v>
       </c>
       <c r="AB165" t="n">
-        <v>9.439017599914223</v>
+        <v>7.873614699696191</v>
       </c>
       <c r="AE165" t="n">
         <v>32</v>
@@ -18653,13 +18653,13 @@
         <v>0.0912631000392139</v>
       </c>
       <c r="Z166" t="n">
-        <v>0.6813575001433492</v>
+        <v>0.03025750024244189</v>
       </c>
       <c r="AA166" t="n">
         <v>9.119395500048995</v>
       </c>
       <c r="AB166" t="n">
-        <v>9.91042280010879</v>
+        <v>9.259322800207883</v>
       </c>
       <c r="AE166" t="n">
         <v>19</v>
@@ -18774,13 +18774,13 @@
         <v>0.06387090031057596</v>
       </c>
       <c r="Z167" t="n">
-        <v>1.833001700229943</v>
+        <v>0.02409389987587929</v>
       </c>
       <c r="AA167" t="n">
         <v>10.05340539989993</v>
       </c>
       <c r="AB167" t="n">
-        <v>11.96362010017037</v>
+        <v>10.15471229981631</v>
       </c>
       <c r="AE167" t="n">
         <v>18</v>
@@ -18886,13 +18886,13 @@
         <v>0.08136320067569613</v>
       </c>
       <c r="Z168" t="n">
-        <v>0.2970931995660067</v>
+        <v>0.02523099957033992</v>
       </c>
       <c r="AA168" t="n">
         <v>9.475574099924415</v>
       </c>
       <c r="AB168" t="n">
-        <v>9.862336900085211</v>
+        <v>9.590474700089544</v>
       </c>
       <c r="AE168" t="n">
         <v>19</v>
@@ -19000,13 +19000,13 @@
         <v>0.06537289964035153</v>
       </c>
       <c r="Z169" t="n">
-        <v>0.2619174001738429</v>
+        <v>0.02428610029164702</v>
       </c>
       <c r="AA169" t="n">
         <v>8.338950200006366</v>
       </c>
       <c r="AB169" t="n">
-        <v>8.672510599717498</v>
+        <v>8.434879299835302</v>
       </c>
       <c r="AE169" t="n">
         <v>19</v>
@@ -19122,13 +19122,13 @@
         <v>0.05662029981613159</v>
       </c>
       <c r="Z170" t="n">
-        <v>0.1860514003783464</v>
+        <v>0.0254308000439778</v>
       </c>
       <c r="AA170" t="n">
         <v>11.45424559991807</v>
       </c>
       <c r="AB170" t="n">
-        <v>11.70479560038075</v>
+        <v>11.54417500004638</v>
       </c>
       <c r="AE170" t="n">
         <v>19</v>
@@ -19234,13 +19234,13 @@
         <v>0.08855889970436692</v>
       </c>
       <c r="Z171" t="n">
-        <v>0.3868976002559066</v>
+        <v>0.02487960015423596</v>
       </c>
       <c r="AA171" t="n">
         <v>9.425404499750584</v>
       </c>
       <c r="AB171" t="n">
-        <v>9.915808000136167</v>
+        <v>9.553790000034496</v>
       </c>
       <c r="AE171" t="n">
         <v>29</v>
@@ -19343,13 +19343,13 @@
         <v>0.04029270028695464</v>
       </c>
       <c r="Z172" t="n">
-        <v>0.1901521999388933</v>
+        <v>0.02560109994374216</v>
       </c>
       <c r="AA172" t="n">
         <v>4.813713400159031</v>
       </c>
       <c r="AB172" t="n">
-        <v>5.051150999963284</v>
+        <v>4.886599899968132</v>
       </c>
       <c r="AE172" t="n">
         <v>17</v>
@@ -19452,13 +19452,13 @@
         <v>0.05550149967893958</v>
       </c>
       <c r="Z173" t="n">
-        <v>0.224244300276041</v>
+        <v>0.02639060001820326</v>
       </c>
       <c r="AA173" t="n">
         <v>5.946027599740773</v>
       </c>
       <c r="AB173" t="n">
-        <v>6.238500199746341</v>
+        <v>6.040646499488503</v>
       </c>
       <c r="AE173" t="n">
         <v>28</v>
@@ -19566,13 +19566,13 @@
         <v>0.09767580032348633</v>
       </c>
       <c r="Z174" t="n">
-        <v>0.3935501999221742</v>
+        <v>0.02826729987282306</v>
       </c>
       <c r="AA174" t="n">
         <v>10.77978619979694</v>
       </c>
       <c r="AB174" t="n">
-        <v>11.28397029964253</v>
+        <v>10.91868739959318</v>
       </c>
       <c r="AE174" t="n">
         <v>36</v>
@@ -19680,13 +19680,13 @@
         <v>0.04626940004527569</v>
       </c>
       <c r="Z175" t="n">
-        <v>0.1970600998029113</v>
+        <v>0.02635269984602928</v>
       </c>
       <c r="AA175" t="n">
         <v>9.490635299589485</v>
       </c>
       <c r="AB175" t="n">
-        <v>9.741675300057977</v>
+        <v>9.570967900101095</v>
       </c>
       <c r="AE175" t="n">
         <v>21</v>
@@ -19791,13 +19791,13 @@
         <v>0.0429619001224637</v>
       </c>
       <c r="Z176" t="n">
-        <v>0.1738318996503949</v>
+        <v>0.02377650002017617</v>
       </c>
       <c r="AA176" t="n">
         <v>5.864593199919909</v>
       </c>
       <c r="AB176" t="n">
-        <v>6.091156600043178</v>
+        <v>5.941101200412959</v>
       </c>
       <c r="AE176" t="n">
         <v>20</v>
@@ -19900,13 +19900,13 @@
         <v>0.06677599949762225</v>
       </c>
       <c r="Z177" t="n">
-        <v>0.2146393000148237</v>
+        <v>0.02871750039048493</v>
       </c>
       <c r="AA177" t="n">
         <v>5.517347699962556</v>
       </c>
       <c r="AB177" t="n">
-        <v>5.808252200018615</v>
+        <v>5.622330400394276</v>
       </c>
       <c r="AE177" t="n">
         <v>19</v>
@@ -20009,13 +20009,13 @@
         <v>0.05016769981011748</v>
       </c>
       <c r="Z178" t="n">
-        <v>0.3256512000225484</v>
+        <v>0.02539419976528734</v>
       </c>
       <c r="AA178" t="n">
         <v>5.071822199970484</v>
       </c>
       <c r="AB178" t="n">
-        <v>5.45965120010078</v>
+        <v>5.159394199843518</v>
       </c>
       <c r="AE178" t="n">
         <v>21</v>
@@ -20118,13 +20118,13 @@
         <v>0.08610700024291873</v>
       </c>
       <c r="Z179" t="n">
-        <v>0.5586947002448142</v>
+        <v>0.03391950018703938</v>
       </c>
       <c r="AA179" t="n">
         <v>5.585006899666041</v>
       </c>
       <c r="AB179" t="n">
-        <v>6.245300900191069</v>
+        <v>5.720525700133294</v>
       </c>
       <c r="AE179" t="n">
         <v>17</v>
@@ -20227,13 +20227,13 @@
         <v>0.08615500014275312</v>
       </c>
       <c r="Z180" t="n">
-        <v>0.5147300995886326</v>
+        <v>0.02318599983118474</v>
       </c>
       <c r="AA180" t="n">
         <v>6.421987900044769</v>
       </c>
       <c r="AB180" t="n">
-        <v>7.036750200204551</v>
+        <v>6.545206100447103</v>
       </c>
       <c r="AE180" t="n">
         <v>17</v>
@@ -20349,13 +20349,13 @@
         <v>0.08337460039183497</v>
       </c>
       <c r="Z181" t="n">
-        <v>0.2890129000879824</v>
+        <v>0.03361590020358562</v>
       </c>
       <c r="AA181" t="n">
         <v>10.87438039993867</v>
       </c>
       <c r="AB181" t="n">
-        <v>11.26241520000622</v>
+        <v>11.00701820012182</v>
       </c>
       <c r="AE181" t="n">
         <v>18</v>
@@ -20462,13 +20462,13 @@
         <v>0.04443279979750514</v>
       </c>
       <c r="Z182" t="n">
-        <v>0.2670104000717402</v>
+        <v>0.0276971998391673</v>
       </c>
       <c r="AA182" t="n">
         <v>11.80714929988608</v>
       </c>
       <c r="AB182" t="n">
-        <v>12.12522620009258</v>
+        <v>11.88591299986001</v>
       </c>
       <c r="AE182" t="n">
         <v>33</v>
@@ -20576,13 +20576,13 @@
         <v>0.04177589993923903</v>
       </c>
       <c r="Z183" t="n">
-        <v>0.170371700078249</v>
+        <v>0.02442600019276142</v>
       </c>
       <c r="AA183" t="n">
         <v>8.641310300212353</v>
       </c>
       <c r="AB183" t="n">
-        <v>8.860036400146782</v>
+        <v>8.714090700261295</v>
       </c>
       <c r="AE183" t="n">
         <v>19</v>
@@ -20697,13 +20697,13 @@
         <v>0.03771730046719313</v>
       </c>
       <c r="Z184" t="n">
-        <v>0.1608767998404801</v>
+        <v>0.02375689963810146</v>
       </c>
       <c r="AA184" t="n">
         <v>9.280183499678969</v>
       </c>
       <c r="AB184" t="n">
-        <v>9.485684199724346</v>
+        <v>9.348564299521968</v>
       </c>
       <c r="AE184" t="n">
         <v>17</v>
@@ -20806,13 +20806,13 @@
         <v>0.0374343004077673</v>
       </c>
       <c r="Z185" t="n">
-        <v>0.1784450002014637</v>
+        <v>0.02495070011354983</v>
       </c>
       <c r="AA185" t="n">
         <v>5.398533899802715</v>
       </c>
       <c r="AB185" t="n">
-        <v>5.62979430006817</v>
+        <v>5.476299999980256</v>
       </c>
       <c r="AE185" t="n">
         <v>18</v>
@@ -20915,13 +20915,13 @@
         <v>0.07395350001752377</v>
       </c>
       <c r="Z186" t="n">
-        <v>0.2590890997089446</v>
+        <v>0.0264950996497646</v>
       </c>
       <c r="AA186" t="n">
         <v>5.403837400022894</v>
       </c>
       <c r="AB186" t="n">
-        <v>5.748254300095141</v>
+        <v>5.515660300035961</v>
       </c>
       <c r="AE186" t="n">
         <v>18</v>
@@ -21033,13 +21033,13 @@
         <v>0.09471199987456203</v>
       </c>
       <c r="Z187" t="n">
-        <v>0.7167711998336017</v>
+        <v>0.02671760006342083</v>
       </c>
       <c r="AA187" t="n">
         <v>13.09904529992491</v>
       </c>
       <c r="AB187" t="n">
-        <v>13.91942079970613</v>
+        <v>13.22936719993595</v>
       </c>
       <c r="AE187" t="n">
         <v>20</v>
@@ -21142,13 +21142,13 @@
         <v>0.040191899985075</v>
       </c>
       <c r="Z188" t="n">
-        <v>0.1746114999987185</v>
+        <v>0.02712409966625273</v>
       </c>
       <c r="AA188" t="n">
         <v>6.230083699803799</v>
       </c>
       <c r="AB188" t="n">
-        <v>6.451330999843776</v>
+        <v>6.30384359951131</v>
       </c>
       <c r="AE188" t="n">
         <v>17</v>
@@ -21251,13 +21251,13 @@
         <v>0.05049159936606884</v>
       </c>
       <c r="Z189" t="n">
-        <v>0.1831648000515997</v>
+        <v>0.02865300013218075</v>
       </c>
       <c r="AA189" t="n">
         <v>6.268401899840683</v>
       </c>
       <c r="AB189" t="n">
-        <v>6.514034199994057</v>
+        <v>6.359522400074638</v>
       </c>
       <c r="AE189" t="n">
         <v>18</v>
@@ -21370,13 +21370,13 @@
         <v>0.06500629987567663</v>
       </c>
       <c r="Z190" t="n">
-        <v>0.2995390999130905</v>
+        <v>0.02420149988029152</v>
       </c>
       <c r="AA190" t="n">
         <v>13.11249809991568</v>
       </c>
       <c r="AB190" t="n">
-        <v>13.48440420022234</v>
+        <v>13.20906660018954</v>
       </c>
       <c r="AE190" t="n">
         <v>24</v>
@@ -21494,13 +21494,13 @@
         <v>0.07007870031520724</v>
       </c>
       <c r="Z191" t="n">
-        <v>0.270134299993515</v>
+        <v>0.02359540003817528</v>
       </c>
       <c r="AA191" t="n">
         <v>8.137327599804848</v>
       </c>
       <c r="AB191" t="n">
-        <v>8.486539300065488</v>
+        <v>8.240000400110148</v>
       </c>
       <c r="AE191" t="n">
         <v>22</v>
@@ -21603,13 +21603,13 @@
         <v>0.0409550997428596</v>
       </c>
       <c r="Z192" t="n">
-        <v>0.1857553999871016</v>
+        <v>0.02515910018701106</v>
       </c>
       <c r="AA192" t="n">
         <v>4.636942700017244</v>
       </c>
       <c r="AB192" t="n">
-        <v>4.872096499893814</v>
+        <v>4.711500200093724</v>
       </c>
       <c r="AE192" t="n">
         <v>21</v>
@@ -21723,13 +21723,13 @@
         <v>0.07715939963236451</v>
       </c>
       <c r="Z193" t="n">
-        <v>0.4006300000473857</v>
+        <v>0.02803940023295581</v>
       </c>
       <c r="AA193" t="n">
         <v>9.220219899900258</v>
       </c>
       <c r="AB193" t="n">
-        <v>9.70713169965893</v>
+        <v>9.3345410998445</v>
       </c>
       <c r="AE193" t="n">
         <v>23</v>
@@ -21843,13 +21843,13 @@
         <v>0.03623649943619967</v>
       </c>
       <c r="Z194" t="n">
-        <v>0.1866790000349283</v>
+        <v>0.02760670019779354</v>
       </c>
       <c r="AA194" t="n">
         <v>6.965589200146496</v>
       </c>
       <c r="AB194" t="n">
-        <v>7.196341699920595</v>
+        <v>7.03726940008346</v>
       </c>
       <c r="AE194" t="n">
         <v>22</v>
@@ -21952,13 +21952,13 @@
         <v>0.04777480009943247</v>
       </c>
       <c r="Z195" t="n">
-        <v>0.2057202002033591</v>
+        <v>0.02869980013929307</v>
       </c>
       <c r="AA195" t="n">
         <v>7.079359299968928</v>
       </c>
       <c r="AB195" t="n">
-        <v>7.342654099687934</v>
+        <v>7.165633699623868</v>
       </c>
       <c r="AE195" t="n">
         <v>23</v>
@@ -22061,13 +22061,13 @@
         <v>0.04317690012976527</v>
       </c>
       <c r="Z196" t="n">
-        <v>0.209429900161922</v>
+        <v>0.02789710008073598</v>
       </c>
       <c r="AA196" t="n">
         <v>7.067985499743372</v>
       </c>
       <c r="AB196" t="n">
-        <v>7.328426899854094</v>
+        <v>7.146894099772908</v>
       </c>
       <c r="AE196" t="n">
         <v>23</v>
@@ -22179,13 +22179,13 @@
         <v>0.08453750004991889</v>
       </c>
       <c r="Z197" t="n">
-        <v>0.2508207000792027</v>
+        <v>0.02776810002978891</v>
       </c>
       <c r="AA197" t="n">
         <v>5.743300199974328</v>
       </c>
       <c r="AB197" t="n">
-        <v>6.085651099681854</v>
+        <v>5.862598499632441</v>
       </c>
       <c r="AE197" t="n">
         <v>21</v>
@@ -22288,13 +22288,13 @@
         <v>0.03840170009061694</v>
       </c>
       <c r="Z198" t="n">
-        <v>0.1774535998702049</v>
+        <v>0.0278288999106735</v>
       </c>
       <c r="AA198" t="n">
         <v>4.863938599824905</v>
       </c>
       <c r="AB198" t="n">
-        <v>5.087677100207657</v>
+        <v>4.938052400248125</v>
       </c>
       <c r="AE198" t="n">
         <v>21</v>
@@ -22397,13 +22397,13 @@
         <v>0.06264410028234124</v>
       </c>
       <c r="Z199" t="n">
-        <v>0.215921999886632</v>
+        <v>0.03310989984311163</v>
       </c>
       <c r="AA199" t="n">
         <v>4.968827699776739</v>
       </c>
       <c r="AB199" t="n">
-        <v>5.253427400253713</v>
+        <v>5.070615300210193</v>
       </c>
       <c r="AE199" t="n">
         <v>21</v>
@@ -22507,13 +22507,13 @@
         <v>0.03572330018505454</v>
       </c>
       <c r="Z200" t="n">
-        <v>0.2039807997643948</v>
+        <v>0.02453759999480098</v>
       </c>
       <c r="AA200" t="n">
         <v>7.543280499987304</v>
       </c>
       <c r="AB200" t="n">
-        <v>7.7925657001324</v>
+        <v>7.613122500362806</v>
       </c>
       <c r="AE200" t="n">
         <v>24</v>
@@ -22616,13 +22616,13 @@
         <v>0.04650120018050075</v>
       </c>
       <c r="Z201" t="n">
-        <v>0.195144500117749</v>
+        <v>0.02873619995079935</v>
       </c>
       <c r="AA201" t="n">
         <v>7.439801999833435</v>
       </c>
       <c r="AB201" t="n">
-        <v>7.689826600253582</v>
+        <v>7.523418300086632</v>
       </c>
       <c r="AE201" t="n">
         <v>23</v>
@@ -22729,13 +22729,13 @@
         <v>20.10597170004621</v>
       </c>
       <c r="Z202" t="n">
-        <v>8.508313900791109</v>
+        <v>0.2610849002376199</v>
       </c>
       <c r="AA202" t="n">
         <v>16.36689080006909</v>
       </c>
       <c r="AB202" t="n">
-        <v>53.86474210082088</v>
+        <v>45.61751310026739</v>
       </c>
       <c r="AC202" t="n">
         <v>5272</v>
@@ -22848,13 +22848,13 @@
         <v>15.19315659999847</v>
       </c>
       <c r="Z203" t="n">
-        <v>3.641991801094264</v>
+        <v>0.2274743006564677</v>
       </c>
       <c r="AA203" t="n">
         <v>13.64772180002183</v>
       </c>
       <c r="AB203" t="n">
-        <v>39.19090580102056</v>
+        <v>35.77638830058277</v>
       </c>
       <c r="AC203" t="n">
         <v>2067</v>
@@ -22966,13 +22966,13 @@
         <v>14.70663239993155</v>
       </c>
       <c r="Z204" t="n">
-        <v>3.622218298725784</v>
+        <v>0.2257596995914355</v>
       </c>
       <c r="AA204" t="n">
         <v>13.99741159996483</v>
       </c>
       <c r="AB204" t="n">
-        <v>46.77719119866379</v>
+        <v>43.38073259952944</v>
       </c>
       <c r="AC204" t="n">
         <v>2068</v>
@@ -23089,13 +23089,13 @@
         <v>11.80691689997911</v>
       </c>
       <c r="Z205" t="n">
-        <v>5.865773399360478</v>
+        <v>0.3518765006447211</v>
       </c>
       <c r="AA205" t="n">
         <v>16.82163170003332</v>
       </c>
       <c r="AB205" t="n">
-        <v>49.21035789931193</v>
+        <v>43.69646100059617</v>
       </c>
       <c r="AC205" t="n">
         <v>2066</v>
@@ -23215,13 +23215,13 @@
         <v>16.64241990027949</v>
       </c>
       <c r="Z206" t="n">
-        <v>3.208013800438493</v>
+        <v>0.306033399538137</v>
       </c>
       <c r="AA206" t="n">
         <v>16.88067260000389</v>
       </c>
       <c r="AB206" t="n">
-        <v>51.53267500072252</v>
+        <v>48.63069459982216</v>
       </c>
       <c r="AC206" t="n">
         <v>5110</v>
@@ -23336,13 +23336,13 @@
         <v>16.48198439972475</v>
       </c>
       <c r="Z207" t="n">
-        <v>4.332460100762546</v>
+        <v>0.3337619006633759</v>
       </c>
       <c r="AA207" t="n">
         <v>12.57397279993165</v>
       </c>
       <c r="AB207" t="n">
-        <v>41.16710230056196</v>
+        <v>37.16840410046279</v>
       </c>
       <c r="AC207" t="n">
         <v>2069</v>
@@ -23455,13 +23455,13 @@
         <v>7.620915299747139</v>
       </c>
       <c r="Z208" t="n">
-        <v>6.036783600691706</v>
+        <v>0.3646157007897273</v>
       </c>
       <c r="AA208" t="n">
         <v>12.77129069995135</v>
       </c>
       <c r="AB208" t="n">
-        <v>35.20217240042984</v>
+        <v>29.53000450052787</v>
       </c>
       <c r="AC208" t="n">
         <v>2079</v>
@@ -23574,13 +23574,13 @@
         <v>13.27123059984297</v>
       </c>
       <c r="Z209" t="n">
-        <v>3.408620398957282</v>
+        <v>0.2716302984626964</v>
       </c>
       <c r="AA209" t="n">
         <v>11.56763280008454</v>
       </c>
       <c r="AB209" t="n">
-        <v>35.12801959877834</v>
+        <v>31.99102949828375</v>
       </c>
       <c r="AC209" t="n">
         <v>2064</v>
@@ -23692,13 +23692,13 @@
         <v>8.987940199673176</v>
       </c>
       <c r="Z210" t="n">
-        <v>2.321429099887609</v>
+        <v>0.1704100001370534</v>
       </c>
       <c r="AA210" t="n">
         <v>14.42125290003605</v>
       </c>
       <c r="AB210" t="n">
-        <v>37.96678099955898</v>
+        <v>35.81576189980842</v>
       </c>
       <c r="AC210" t="n">
         <v>2060</v>
@@ -23810,13 +23810,13 @@
         <v>11.04384359996766</v>
       </c>
       <c r="Z211" t="n">
-        <v>2.314997800160199</v>
+        <v>0.178752800100483</v>
       </c>
       <c r="AA211" t="n">
         <v>12.9980848999694</v>
       </c>
       <c r="AB211" t="n">
-        <v>39.00566620018799</v>
+        <v>36.86942120012827</v>
       </c>
       <c r="AC211" t="n">
         <v>2062</v>
@@ -23934,13 +23934,13 @@
         <v>13.11727110017091</v>
       </c>
       <c r="Z212" t="n">
-        <v>4.113195799756795</v>
+        <v>0.2418647009180859</v>
       </c>
       <c r="AA212" t="n">
         <v>15.12969249999151</v>
       </c>
       <c r="AB212" t="n">
-        <v>45.55374240002129</v>
+        <v>41.68241130118258</v>
       </c>
       <c r="AC212" t="n">
         <v>2079</v>
@@ -24064,13 +24064,13 @@
         <v>5.970233500003815</v>
       </c>
       <c r="Z213" t="n">
-        <v>3.826804300304502</v>
+        <v>0.2790788998827338</v>
       </c>
       <c r="AA213" t="n">
         <v>18.6530973999761</v>
       </c>
       <c r="AB213" t="n">
-        <v>39.81065930030309</v>
+        <v>36.26293389988132</v>
       </c>
       <c r="AC213" t="n">
         <v>2056</v>
@@ -24182,13 +24182,13 @@
         <v>14.7605016999878</v>
       </c>
       <c r="Z214" t="n">
-        <v>1.829104500357062</v>
+        <v>0.1524622997967526</v>
       </c>
       <c r="AA214" t="n">
         <v>12.69074390002061</v>
       </c>
       <c r="AB214" t="n">
-        <v>39.48072770028375</v>
+        <v>37.80408549972344</v>
       </c>
       <c r="AC214" t="n">
         <v>4968</v>
@@ -24310,13 +24310,13 @@
         <v>8.962914399802685</v>
       </c>
       <c r="Z215" t="n">
-        <v>3.909238000866026</v>
+        <v>0.2876645008800551</v>
       </c>
       <c r="AA215" t="n">
         <v>18.30469750007614</v>
       </c>
       <c r="AB215" t="n">
-        <v>40.9171320006717</v>
+        <v>37.29555850068573</v>
       </c>
       <c r="AC215" t="n">
         <v>2054</v>
@@ -24436,13 +24436,13 @@
         <v>26.39673899998888</v>
       </c>
       <c r="Z216" t="n">
-        <v>2.886939399410039</v>
+        <v>0.3099326998926699</v>
       </c>
       <c r="AA216" t="n">
         <v>17.10883739998098</v>
       </c>
       <c r="AB216" t="n">
-        <v>61.0063421993982</v>
+        <v>58.42933549988084</v>
       </c>
       <c r="AC216" t="n">
         <v>9338</v>
@@ -24564,13 +24564,13 @@
         <v>15.99699700018391</v>
       </c>
       <c r="Z217" t="n">
-        <v>2.535339000169188</v>
+        <v>0.245007700403221</v>
       </c>
       <c r="AA217" t="n">
         <v>19.98909369995818</v>
       </c>
       <c r="AB217" t="n">
-        <v>51.71963300032075</v>
+        <v>49.42930170055479</v>
       </c>
       <c r="AC217" t="n">
         <v>2070</v>
@@ -24682,13 +24682,13 @@
         <v>10.84137450018898</v>
       </c>
       <c r="Z218" t="n">
-        <v>2.953380499500781</v>
+        <v>0.2044638992520049</v>
       </c>
       <c r="AA218" t="n">
         <v>15.48108870000578</v>
       </c>
       <c r="AB218" t="n">
-        <v>43.66343429975677</v>
+        <v>40.914517699508</v>
       </c>
       <c r="AC218" t="n">
         <v>2055</v>
@@ -24803,13 +24803,13 @@
         <v>17.68051300011575</v>
       </c>
       <c r="Z219" t="n">
-        <v>3.348934300243855</v>
+        <v>0.1936914997640997</v>
       </c>
       <c r="AA219" t="n">
         <v>12.52802630001679</v>
       </c>
       <c r="AB219" t="n">
-        <v>43.73316450044513</v>
+        <v>40.57792169996537</v>
       </c>
       <c r="AC219" t="n">
         <v>2070</v>
@@ -24922,13 +24922,13 @@
         <v>16.52993339998648</v>
       </c>
       <c r="Z220" t="n">
-        <v>3.090420899912715</v>
+        <v>0.2421855990542099</v>
       </c>
       <c r="AA220" t="n">
         <v>11.65550840005744</v>
       </c>
       <c r="AB220" t="n">
-        <v>40.53025329986122</v>
+        <v>37.68201799900271</v>
       </c>
       <c r="AC220" t="n">
         <v>5089</v>
@@ -25049,13 +25049,13 @@
         <v>6.374825599603355</v>
       </c>
       <c r="Z221" t="n">
-        <v>4.038319599349052</v>
+        <v>0.2316601995844394</v>
       </c>
       <c r="AA221" t="n">
         <v>14.01195680000819</v>
       </c>
       <c r="AB221" t="n">
-        <v>34.14693849894684</v>
+        <v>30.34027909918223</v>
       </c>
       <c r="AC221" t="n">
         <v>2056</v>
@@ -25175,13 +25175,13 @@
         <v>7.916779899969697</v>
       </c>
       <c r="Z222" t="n">
-        <v>3.777922099921852</v>
+        <v>0.216469700797461</v>
       </c>
       <c r="AA222" t="n">
         <v>18.71938909997698</v>
       </c>
       <c r="AB222" t="n">
-        <v>43.36042679985985</v>
+        <v>39.79897440073546</v>
       </c>
       <c r="AC222" t="n">
         <v>2067</v>
@@ -25313,13 +25313,13 @@
         <v>10.05892849992961</v>
       </c>
       <c r="Z223" t="n">
-        <v>3.040546400472522</v>
+        <v>0.2379596001701429</v>
       </c>
       <c r="AA223" t="n">
         <v>19.86496030003764</v>
       </c>
       <c r="AB223" t="n">
-        <v>46.19675020046998</v>
+        <v>43.3941634001676</v>
       </c>
       <c r="AC223" t="n">
         <v>4444</v>
@@ -25431,13 +25431,13 @@
         <v>17.54849549988285</v>
       </c>
       <c r="Z224" t="n">
-        <v>1.966508600395173</v>
+        <v>0.1913147999439389</v>
       </c>
       <c r="AA224" t="n">
         <v>13.34001520008314</v>
       </c>
       <c r="AB224" t="n">
-        <v>45.49242520029657</v>
+        <v>43.71723139984533</v>
       </c>
       <c r="AC224" t="n">
         <v>7570</v>
@@ -25560,13 +25560,13 @@
         <v>11.71755180042237</v>
       </c>
       <c r="Z225" t="n">
-        <v>2.39506410015747</v>
+        <v>0.1466174991801381</v>
       </c>
       <c r="AA225" t="n">
         <v>15.40420909994282</v>
       </c>
       <c r="AB225" t="n">
-        <v>40.09807690058369</v>
+        <v>37.84963029960636</v>
       </c>
       <c r="AC225" t="n">
         <v>2053</v>
@@ -25679,13 +25679,13 @@
         <v>12.99753989977762</v>
       </c>
       <c r="Z226" t="n">
-        <v>2.491015700157732</v>
+        <v>0.1537671991391107</v>
       </c>
       <c r="AA226" t="n">
         <v>15.20640599995386</v>
       </c>
       <c r="AB226" t="n">
-        <v>37.02156639995519</v>
+        <v>34.68431789893657</v>
       </c>
       <c r="AC226" t="n">
         <v>4659</v>
@@ -25803,13 +25803,13 @@
         <v>15.26203250000253</v>
       </c>
       <c r="Z227" t="n">
-        <v>2.990197100210935</v>
+        <v>0.3353677015984431</v>
       </c>
       <c r="AA227" t="n">
         <v>17.42006629996467</v>
       </c>
       <c r="AB227" t="n">
-        <v>45.1293777001556</v>
+        <v>42.47454830154311</v>
       </c>
       <c r="AC227" t="n">
         <v>5108</v>
@@ -25930,13 +25930,13 @@
         <v>9.171779800206423</v>
       </c>
       <c r="Z228" t="n">
-        <v>3.181223298888654</v>
+        <v>0.2312273998977616</v>
       </c>
       <c r="AA228" t="n">
         <v>14.67781749996357</v>
       </c>
       <c r="AB228" t="n">
-        <v>36.73004779906478</v>
+        <v>33.78005190007389</v>
       </c>
       <c r="AC228" t="n">
         <v>2052</v>
@@ -26054,13 +26054,13 @@
         <v>19.49453520029783</v>
       </c>
       <c r="Z229" t="n">
-        <v>2.437299500219524</v>
+        <v>0.1556898002745584</v>
       </c>
       <c r="AA229" t="n">
         <v>11.75589309993666</v>
       </c>
       <c r="AB229" t="n">
-        <v>35.01475890050642</v>
+        <v>32.73314920056146</v>
       </c>
       <c r="AC229" t="n">
         <v>2058</v>
@@ -26176,13 +26176,13 @@
         <v>14.63708010036498</v>
       </c>
       <c r="Z230" t="n">
-        <v>3.032620499376208</v>
+        <v>0.2186750996625051</v>
       </c>
       <c r="AA230" t="n">
         <v>10.58981719997246</v>
       </c>
       <c r="AB230" t="n">
-        <v>32.0026533997152</v>
+        <v>29.1887080000015</v>
       </c>
       <c r="AC230" t="n">
         <v>2056</v>
@@ -26299,13 +26299,13 @@
         <v>12.45930070010945</v>
       </c>
       <c r="Z231" t="n">
-        <v>3.298506098799407</v>
+        <v>0.1933422989677638</v>
       </c>
       <c r="AA231" t="n">
         <v>11.65003440005239</v>
       </c>
       <c r="AB231" t="n">
-        <v>31.60006369894836</v>
+        <v>28.49489989911672</v>
       </c>
       <c r="AC231" t="n">
         <v>2077</v>
@@ -26428,13 +26428,13 @@
         <v>6.1897539999336</v>
       </c>
       <c r="Z232" t="n">
-        <v>3.901212400291115</v>
+        <v>0.2416357001056895</v>
       </c>
       <c r="AA232" t="n">
         <v>17.16871900006663</v>
       </c>
       <c r="AB232" t="n">
-        <v>33.48070750024635</v>
+        <v>29.82113080006093</v>
       </c>
       <c r="AC232" t="n">
         <v>2058</v>
@@ -26548,13 +26548,13 @@
         <v>12.80049529997632</v>
       </c>
       <c r="Z233" t="n">
-        <v>4.317567800637335</v>
+        <v>0.2761278988327831</v>
       </c>
       <c r="AA233" t="n">
         <v>12.69652380002663</v>
       </c>
       <c r="AB233" t="n">
-        <v>34.58032620069571</v>
+        <v>30.53888629889116</v>
       </c>
       <c r="AC233" t="n">
         <v>2066</v>
@@ -26673,13 +26673,13 @@
         <v>11.18074769992381</v>
       </c>
       <c r="Z234" t="n">
-        <v>2.026627200189978</v>
+        <v>0.1673243994591758</v>
       </c>
       <c r="AA234" t="n">
         <v>15.78134259989019</v>
       </c>
       <c r="AB234" t="n">
-        <v>34.47909700009041</v>
+        <v>32.6197941993596</v>
       </c>
       <c r="AC234" t="n">
         <v>2059</v>
@@ -26799,13 +26799,13 @@
         <v>16.09692140016705</v>
       </c>
       <c r="Z235" t="n">
-        <v>2.647415300365537</v>
+        <v>0.1743786000879481</v>
       </c>
       <c r="AA235" t="n">
         <v>14.95732080005109</v>
       </c>
       <c r="AB235" t="n">
-        <v>38.34569910052232</v>
+        <v>35.87266240024474</v>
       </c>
       <c r="AC235" t="n">
         <v>4823</v>
@@ -26924,13 +26924,13 @@
         <v>15.07731570024043</v>
       </c>
       <c r="Z236" t="n">
-        <v>4.320027499925345</v>
+        <v>0.2006318991770968</v>
       </c>
       <c r="AA236" t="n">
         <v>13.87672359996941</v>
       </c>
       <c r="AB236" t="n">
-        <v>38.36119370022789</v>
+        <v>34.24179809947964</v>
       </c>
       <c r="AC236" t="n">
         <v>2075</v>
@@ -27046,13 +27046,13 @@
         <v>25.3566740998067</v>
       </c>
       <c r="Z237" t="n">
-        <v>3.258336901199073</v>
+        <v>0.3581816996447742</v>
       </c>
       <c r="AA237" t="n">
         <v>15.1940939000342</v>
       </c>
       <c r="AB237" t="n">
-        <v>48.71907220105641</v>
+        <v>45.81891699950211</v>
       </c>
       <c r="AC237" t="n">
         <v>8708</v>
@@ -27166,13 +27166,13 @@
         <v>15.51890020025894</v>
       </c>
       <c r="Z238" t="n">
-        <v>3.106476199813187</v>
+        <v>0.2452961002709344</v>
       </c>
       <c r="AA238" t="n">
         <v>12.8496156000765</v>
       </c>
       <c r="AB238" t="n">
-        <v>37.46839180006646</v>
+        <v>34.6072117005242</v>
       </c>
       <c r="AC238" t="n">
         <v>5076</v>
@@ -27289,13 +27289,13 @@
         <v>30.10339360032231</v>
       </c>
       <c r="Z239" t="n">
-        <v>2.280535000376403</v>
+        <v>0.1519507998600602</v>
       </c>
       <c r="AA239" t="n">
         <v>13.86644220002927</v>
       </c>
       <c r="AB239" t="n">
-        <v>50.40369560068939</v>
+        <v>48.27511140017305</v>
       </c>
       <c r="AC239" t="n">
         <v>12453</v>
@@ -27414,13 +27414,13 @@
         <v>19.25449179997668</v>
       </c>
       <c r="Z240" t="n">
-        <v>4.75878900103271</v>
+        <v>0.3445986001752317</v>
       </c>
       <c r="AA240" t="n">
         <v>15.90942709997762</v>
       </c>
       <c r="AB240" t="n">
-        <v>45.91180550097488</v>
+        <v>41.4976151001174</v>
       </c>
       <c r="AC240" t="n">
         <v>5210</v>
@@ -27536,13 +27536,13 @@
         <v>8.093798999674618</v>
       </c>
       <c r="Z241" t="n">
-        <v>2.392027199734002</v>
+        <v>0.1225772997131571</v>
       </c>
       <c r="AA241" t="n">
         <v>14.6145617000293</v>
       </c>
       <c r="AB241" t="n">
-        <v>30.53392539941706</v>
+        <v>28.26447549939621</v>
       </c>
       <c r="AC241" t="n">
         <v>2064</v>
@@ -27657,13 +27657,13 @@
         <v>7.149222100153565</v>
       </c>
       <c r="Z242" t="n">
-        <v>3.533703800290823</v>
+        <v>0.1757820001803339</v>
       </c>
       <c r="AA242" t="n">
         <v>15.07848010002635</v>
       </c>
       <c r="AB242" t="n">
-        <v>31.89432680036407</v>
+        <v>28.53640500025358</v>
       </c>
       <c r="AC242" t="n">
         <v>2084</v>
@@ -27784,13 +27784,13 @@
         <v>6.417862600181252</v>
       </c>
       <c r="Z243" t="n">
-        <v>1.748069600202143</v>
+        <v>0.1173882010625675</v>
       </c>
       <c r="AA243" t="n">
         <v>16.43921800004318</v>
       </c>
       <c r="AB243" t="n">
-        <v>30.51606630044989</v>
+        <v>28.88538490131032</v>
       </c>
       <c r="AC243" t="n">
         <v>2056</v>
@@ -27908,13 +27908,13 @@
         <v>14.09931880002841</v>
       </c>
       <c r="Z244" t="n">
-        <v>2.366355900187045</v>
+        <v>0.1683584995334968</v>
       </c>
       <c r="AA244" t="n">
         <v>16.34346390003338</v>
       </c>
       <c r="AB244" t="n">
-        <v>38.04084400017746</v>
+        <v>35.84284659952391</v>
       </c>
       <c r="AC244" t="n">
         <v>2057</v>
@@ -28026,13 +28026,13 @@
         <v>31.51467399997637</v>
       </c>
       <c r="Z245" t="n">
-        <v>2.875278198625892</v>
+        <v>0.3221458989428356</v>
       </c>
       <c r="AA245" t="n">
         <v>13.38171430001967</v>
       </c>
       <c r="AB245" t="n">
-        <v>52.85681139864028</v>
+        <v>50.30367909895722</v>
       </c>
       <c r="AC245" t="n">
         <v>11967</v>
@@ -28155,13 +28155,13 @@
         <v>10.27147040003911</v>
       </c>
       <c r="Z246" t="n">
-        <v>3.201013001147658</v>
+        <v>0.2094942994881421</v>
       </c>
       <c r="AA246" t="n">
         <v>17.27031330007594</v>
       </c>
       <c r="AB246" t="n">
-        <v>36.51728170120623</v>
+        <v>33.52576299954671</v>
       </c>
       <c r="AC246" t="n">
         <v>2060</v>
@@ -28285,13 +28285,13 @@
         <v>13.42517519975081</v>
       </c>
       <c r="Z247" t="n">
-        <v>2.1424032994546</v>
+        <v>0.1493806000798941</v>
       </c>
       <c r="AA247" t="n">
         <v>14.6962910000002</v>
       </c>
       <c r="AB247" t="n">
-        <v>36.13593289919663</v>
+        <v>34.14291019982193</v>
       </c>
       <c r="AC247" t="n">
         <v>2056</v>
@@ -28405,13 +28405,13 @@
         <v>12.02068149996921</v>
       </c>
       <c r="Z248" t="n">
-        <v>2.273864400107414</v>
+        <v>0.1586046004667878</v>
       </c>
       <c r="AA248" t="n">
         <v>13.94664510001894</v>
       </c>
       <c r="AB248" t="n">
-        <v>35.69998819998</v>
+        <v>33.58472840033937</v>
       </c>
       <c r="AC248" t="n">
         <v>2071</v>
@@ -28523,13 +28523,13 @@
         <v>10.9374429997988</v>
       </c>
       <c r="Z249" t="n">
-        <v>2.942095100414008</v>
+        <v>0.1919735011179</v>
       </c>
       <c r="AA249" t="n">
         <v>15.24576710001566</v>
       </c>
       <c r="AB249" t="n">
-        <v>35.89582770026755</v>
+        <v>33.14570610097144</v>
       </c>
       <c r="AC249" t="n">
         <v>2061</v>
@@ -28645,13 +28645,13 @@
         <v>13.95735230017453</v>
       </c>
       <c r="Z250" t="n">
-        <v>4.086309800855815</v>
+        <v>0.2740285008912906</v>
       </c>
       <c r="AA250" t="n">
         <v>14.36572959995829</v>
       </c>
       <c r="AB250" t="n">
-        <v>38.77189560094848</v>
+        <v>34.95961430098396</v>
       </c>
       <c r="AC250" t="n">
         <v>2083</v>
@@ -28765,13 +28765,13 @@
         <v>14.87909029982984</v>
       </c>
       <c r="Z251" t="n">
-        <v>5.748624199535698</v>
+        <v>0.4626159993931651</v>
       </c>
       <c r="AA251" t="n">
         <v>12.97042909997981</v>
       </c>
       <c r="AB251" t="n">
-        <v>40.85275179939345</v>
+        <v>35.56674359925091</v>
       </c>
       <c r="AC251" t="n">
         <v>4646</v>
@@ -28888,13 +28888,13 @@
         <v>5.823845100123435</v>
       </c>
       <c r="Z252" t="n">
-        <v>2.748075698968023</v>
+        <v>0.1733060998376459</v>
       </c>
       <c r="AA252" t="n">
         <v>15.65713089995552</v>
       </c>
       <c r="AB252" t="n">
-        <v>33.89669349906035</v>
+        <v>31.32192389992997</v>
       </c>
       <c r="AC252" t="n">
         <v>2053</v>
@@ -29006,13 +29006,13 @@
         <v>16.99919869983569</v>
       </c>
       <c r="Z253" t="n">
-        <v>3.813441599253565</v>
+        <v>0.2489810996921733</v>
       </c>
       <c r="AA253" t="n">
         <v>13.5307239999529</v>
       </c>
       <c r="AB253" t="n">
-        <v>44.58646249910817</v>
+        <v>41.02200199954677</v>
       </c>
       <c r="AC253" t="n">
         <v>4937</v>
@@ -29127,13 +29127,13 @@
         <v>14.95608000038192</v>
       </c>
       <c r="Z254" t="n">
-        <v>2.367881199810654</v>
+        <v>0.1483775997767225</v>
       </c>
       <c r="AA254" t="n">
         <v>16.54459469998255</v>
       </c>
       <c r="AB254" t="n">
-        <v>44.01157470024191</v>
+        <v>41.79207110020798</v>
       </c>
       <c r="AC254" t="n">
         <v>2068</v>
@@ -29249,13 +29249,13 @@
         <v>14.14839449990541</v>
       </c>
       <c r="Z255" t="n">
-        <v>4.103292700368911</v>
+        <v>0.3113987998804078</v>
       </c>
       <c r="AA255" t="n">
         <v>16.85434159997385</v>
       </c>
       <c r="AB255" t="n">
-        <v>42.89497730031144</v>
+        <v>39.10308339982294</v>
       </c>
       <c r="AC255" t="n">
         <v>2062</v>
@@ -29367,13 +29367,13 @@
         <v>11.24688739981502</v>
       </c>
       <c r="Z256" t="n">
-        <v>2.918661200907081</v>
+        <v>0.1935016004135832</v>
       </c>
       <c r="AA256" t="n">
         <v>13.11819439998362</v>
       </c>
       <c r="AB256" t="n">
-        <v>34.77441680070478</v>
+        <v>32.04925720021129</v>
       </c>
       <c r="AC256" t="n">
         <v>2060</v>
@@ -29488,13 +29488,13 @@
         <v>8.799929200205952</v>
       </c>
       <c r="Z257" t="n">
-        <v>3.98705610120669</v>
+        <v>0.2446517010685056</v>
       </c>
       <c r="AA257" t="n">
         <v>15.21611869998742</v>
       </c>
       <c r="AB257" t="n">
-        <v>35.81219250150025</v>
+        <v>32.06978810136206</v>
       </c>
       <c r="AC257" t="n">
         <v>2050</v>
@@ -29610,13 +29610,13 @@
         <v>10.78989580040798</v>
       </c>
       <c r="Z258" t="n">
-        <v>4.30188970034942</v>
+        <v>0.2858421010896564</v>
       </c>
       <c r="AA258" t="n">
         <v>21.64300739997998</v>
       </c>
       <c r="AB258" t="n">
-        <v>42.85700050077867</v>
+        <v>38.8409529015189</v>
       </c>
       <c r="AC258" t="n">
         <v>2069</v>
@@ -29735,13 +29735,13 @@
         <v>11.04646890005097</v>
       </c>
       <c r="Z259" t="n">
-        <v>2.89940829994157</v>
+        <v>0.1166155003011227</v>
       </c>
       <c r="AA259" t="n">
         <v>15.48691449989565</v>
       </c>
       <c r="AB259" t="n">
-        <v>33.02394350001123</v>
+        <v>30.24115070037078</v>
       </c>
       <c r="AC259" t="n">
         <v>4680</v>
@@ -29863,13 +29863,13 @@
         <v>12.1374723999761</v>
       </c>
       <c r="Z260" t="n">
-        <v>2.432407300919294</v>
+        <v>0.2046667010290548</v>
       </c>
       <c r="AA260" t="n">
         <v>17.13687120005488</v>
       </c>
       <c r="AB260" t="n">
-        <v>33.42924060090445</v>
+        <v>31.20150000101421</v>
       </c>
       <c r="AC260" t="n">
         <v>2056</v>
@@ -29987,13 +29987,13 @@
         <v>15.71915070014074</v>
       </c>
       <c r="Z261" t="n">
-        <v>1.230905999429524</v>
+        <v>0.1015080998186022</v>
       </c>
       <c r="AA261" t="n">
         <v>17.51711219991557</v>
       </c>
       <c r="AB261" t="n">
-        <v>37.83877759962343</v>
+        <v>36.70937970001251</v>
       </c>
       <c r="AC261" t="n">
         <v>5013</v>
@@ -30108,13 +30108,13 @@
         <v>13.53074949979782</v>
       </c>
       <c r="Z262" t="n">
-        <v>3.08143669879064</v>
+        <v>0.2508536984678358</v>
       </c>
       <c r="AA262" t="n">
         <v>84.70994890003931</v>
       </c>
       <c r="AB262" t="n">
-        <v>104.918648298597</v>
+        <v>102.0880652982742</v>
       </c>
       <c r="AC262" t="n">
         <v>2061</v>
@@ -30230,13 +30230,13 @@
         <v>13.14402929972857</v>
       </c>
       <c r="Z263" t="n">
-        <v>3.225215000100434</v>
+        <v>0.1897197999060154</v>
       </c>
       <c r="AA263" t="n">
         <v>88.90635090006981</v>
       </c>
       <c r="AB263" t="n">
-        <v>108.6937337998534</v>
+        <v>105.6582385996589</v>
       </c>
       <c r="AC263" t="n">
         <v>2061</v>
@@ -30359,13 +30359,13 @@
         <v>23.59082549996674</v>
       </c>
       <c r="Z264" t="n">
-        <v>3.030179298948497</v>
+        <v>0.3582751987269148</v>
       </c>
       <c r="AA264" t="n">
         <v>94.71349640004337</v>
       </c>
       <c r="AB264" t="n">
-        <v>125.3645984989125</v>
+        <v>122.6926943986909</v>
       </c>
       <c r="AC264" t="n">
         <v>2056</v>
@@ -30482,13 +30482,13 @@
         <v>17.14895089995116</v>
       </c>
       <c r="Z265" t="n">
-        <v>3.098550599534065</v>
+        <v>0.2060357991140336</v>
       </c>
       <c r="AA265" t="n">
         <v>90.28343619999941</v>
       </c>
       <c r="AB265" t="n">
-        <v>115.3670233995654</v>
+        <v>112.4745085991453</v>
       </c>
       <c r="AC265" t="n">
         <v>2079</v>
@@ -30610,13 +30610,13 @@
         <v>14.52985410019755</v>
       </c>
       <c r="Z266" t="n">
-        <v>4.558008900377899</v>
+        <v>0.4001131996046752</v>
       </c>
       <c r="AA266" t="n">
         <v>85.00182460003998</v>
       </c>
       <c r="AB266" t="n">
-        <v>109.2093060006155</v>
+        <v>105.0514102998422</v>
       </c>
       <c r="AC266" t="n">
         <v>2060</v>
@@ -30742,13 +30742,13 @@
         <v>7.91539609991014</v>
       </c>
       <c r="Z267" t="n">
-        <v>1.796315600164235</v>
+        <v>0.1467411000048742</v>
       </c>
       <c r="AA267" t="n">
         <v>29.67639729997609</v>
       </c>
       <c r="AB267" t="n">
-        <v>44.22696190001443</v>
+        <v>42.57738739985507</v>
       </c>
       <c r="AC267" t="n">
         <v>2052</v>
@@ -30864,13 +30864,13 @@
         <v>14.17368909996003</v>
       </c>
       <c r="Z268" t="n">
-        <v>2.270633600186557</v>
+        <v>0.393184199812822</v>
       </c>
       <c r="AA268" t="n">
         <v>24.55446780007333</v>
       </c>
       <c r="AB268" t="n">
-        <v>46.28431220015045</v>
+        <v>44.40686279977672</v>
       </c>
       <c r="AC268" t="n">
         <v>4658</v>
@@ -30992,13 +30992,13 @@
         <v>12.36393099976704</v>
       </c>
       <c r="Z269" t="n">
-        <v>2.357498799450696</v>
+        <v>0.3111968995071948</v>
       </c>
       <c r="AA269" t="n">
         <v>29.1188242000062</v>
       </c>
       <c r="AB269" t="n">
-        <v>48.95741099922452</v>
+        <v>46.91110909928102</v>
       </c>
       <c r="AC269" t="n">
         <v>2054</v>
@@ -31122,13 +31122,13 @@
         <v>34.37051049992442</v>
       </c>
       <c r="Z270" t="n">
-        <v>1.791175400838256</v>
+        <v>0.2594680007314309</v>
       </c>
       <c r="AA270" t="n">
         <v>23.63702050002757</v>
       </c>
       <c r="AB270" t="n">
-        <v>66.78188170073554</v>
+        <v>65.25017430062871</v>
       </c>
       <c r="AC270" t="n">
         <v>17290</v>
@@ -31242,13 +31242,13 @@
         <v>9.623882499989122</v>
       </c>
       <c r="Z271" t="n">
-        <v>3.401672699954361</v>
+        <v>0.3033841002034023</v>
       </c>
       <c r="AA271" t="n">
         <v>86.29176139994524</v>
       </c>
       <c r="AB271" t="n">
-        <v>104.8431778999511</v>
+        <v>101.7448893002002</v>
       </c>
       <c r="AC271" t="n">
         <v>4368</v>
@@ -31360,13 +31360,13 @@
         <v>14.65754339983687</v>
       </c>
       <c r="Z272" t="n">
-        <v>1.394445099402219</v>
+        <v>0.1591349997324869</v>
       </c>
       <c r="AA272" t="n">
         <v>22.70713120000437</v>
       </c>
       <c r="AB272" t="n">
-        <v>43.51796869921964</v>
+        <v>42.2826585995499</v>
       </c>
       <c r="AC272" t="n">
         <v>2058</v>
@@ -31484,13 +31484,13 @@
         <v>13.99111359985545</v>
       </c>
       <c r="Z273" t="n">
-        <v>2.047820700332522</v>
+        <v>0.168751499732025</v>
       </c>
       <c r="AA273" t="n">
         <v>54.73385299998336</v>
       </c>
       <c r="AB273" t="n">
-        <v>75.04318760021124</v>
+        <v>73.16411839961074</v>
       </c>
       <c r="AC273" t="n">
         <v>2077</v>
@@ -31602,13 +31602,13 @@
         <v>13.63822000008076</v>
       </c>
       <c r="Z274" t="n">
-        <v>2.248627699445933</v>
+        <v>0.1985730992164463</v>
       </c>
       <c r="AA274" t="n">
         <v>17.99334729998372</v>
       </c>
       <c r="AB274" t="n">
-        <v>39.85840569948778</v>
+        <v>37.80835109925829</v>
       </c>
       <c r="AC274" t="n">
         <v>2091</v>
@@ -31727,13 +31727,13 @@
         <v>10.57756489980966</v>
       </c>
       <c r="Z275" t="n">
-        <v>3.837001000065356</v>
+        <v>0.3128644002135843</v>
       </c>
       <c r="AA275" t="n">
         <v>20.36690839997027</v>
       </c>
       <c r="AB275" t="n">
-        <v>40.60393129987642</v>
+        <v>37.07979470002465</v>
       </c>
       <c r="AC275" t="n">
         <v>2062</v>
@@ -31852,13 +31852,13 @@
         <v>8.647497800178826</v>
       </c>
       <c r="Z276" t="n">
-        <v>1.256435399875045</v>
+        <v>0.08334130013827235</v>
       </c>
       <c r="AA276" t="n">
         <v>19.10453089990187</v>
       </c>
       <c r="AB276" t="n">
-        <v>32.97997109999415</v>
+        <v>31.80687700025737</v>
       </c>
       <c r="AC276" t="n">
         <v>2061</v>
@@ -31982,13 +31982,13 @@
         <v>6.828543799929321</v>
       </c>
       <c r="Z277" t="n">
-        <v>2.31603639991954</v>
+        <v>0.1698623000411317</v>
       </c>
       <c r="AA277" t="n">
         <v>98.73346349992789</v>
       </c>
       <c r="AB277" t="n">
-        <v>111.6270299998578</v>
+        <v>109.4808558999794</v>
       </c>
       <c r="AC277" t="n">
         <v>2060</v>
@@ -32100,13 +32100,13 @@
         <v>6.005569499917328</v>
       </c>
       <c r="Z278" t="n">
-        <v>1.88852220075205</v>
+        <v>0.1298195002600551</v>
       </c>
       <c r="AA278" t="n">
         <v>17.70402899989858</v>
       </c>
       <c r="AB278" t="n">
-        <v>29.14746020059101</v>
+        <v>27.38875750009902</v>
       </c>
       <c r="AC278" t="n">
         <v>2060</v>
@@ -32218,13 +32218,13 @@
         <v>10.37432580022141</v>
       </c>
       <c r="Z279" t="n">
-        <v>1.623338100500405</v>
+        <v>0.08448590035550296</v>
       </c>
       <c r="AA279" t="n">
         <v>19.36912420007866</v>
       </c>
       <c r="AB279" t="n">
-        <v>34.79601100075524</v>
+        <v>33.25715880061034</v>
       </c>
       <c r="AC279" t="n">
         <v>2059</v>
@@ -32336,13 +32336,13 @@
         <v>12.65533510036767</v>
       </c>
       <c r="Z280" t="n">
-        <v>0.4833164000883698</v>
+        <v>0.07110379985533655</v>
       </c>
       <c r="AA280" t="n">
         <v>17.3839196000481</v>
       </c>
       <c r="AB280" t="n">
-        <v>33.7368765004212</v>
+        <v>33.32466390018817</v>
       </c>
       <c r="AC280" t="n">
         <v>4685</v>
@@ -32464,13 +32464,13 @@
         <v>10.70271460013464</v>
       </c>
       <c r="Z281" t="n">
-        <v>3.192703399341553</v>
+        <v>0.2847566994605586</v>
       </c>
       <c r="AA281" t="n">
         <v>17.1154825000558</v>
       </c>
       <c r="AB281" t="n">
-        <v>33.66453409940004</v>
+        <v>30.75658739951905</v>
       </c>
       <c r="AC281" t="n">
         <v>2057</v>
@@ -32584,13 +32584,13 @@
         <v>13.86097340006381</v>
       </c>
       <c r="Z282" t="n">
-        <v>3.504884300287813</v>
+        <v>0.32934709941037</v>
       </c>
       <c r="AA282" t="n">
         <v>14.65281759994105</v>
       </c>
       <c r="AB282" t="n">
-        <v>36.18003260041587</v>
+        <v>33.00449539953843</v>
       </c>
       <c r="AC282" t="n">
         <v>2081</v>
@@ -32706,13 +32706,13 @@
         <v>19.17686750041321</v>
       </c>
       <c r="Z283" t="n">
-        <v>0.9969574995338917</v>
+        <v>0.1166175997350365</v>
       </c>
       <c r="AA283" t="n">
         <v>14.52014859998599</v>
       </c>
       <c r="AB283" t="n">
-        <v>37.74204459984321</v>
+        <v>36.86170470004436</v>
       </c>
       <c r="AC283" t="n">
         <v>5264</v>
@@ -32833,13 +32833,13 @@
         <v>10.91742300009355</v>
       </c>
       <c r="Z284" t="n">
-        <v>3.291124899871647</v>
+        <v>0.2569893999025226</v>
       </c>
       <c r="AA284" t="n">
         <v>14.63002360006794</v>
       </c>
       <c r="AB284" t="n">
-        <v>32.15569929999765</v>
+        <v>29.12156380002853</v>
       </c>
       <c r="AC284" t="n">
         <v>4592</v>
@@ -32951,13 +32951,13 @@
         <v>20.11515789991245</v>
       </c>
       <c r="Z285" t="n">
-        <v>1.415616599842906</v>
+        <v>0.08330909942742437</v>
       </c>
       <c r="AA285" t="n">
         <v>15.15942350006662</v>
       </c>
       <c r="AB285" t="n">
-        <v>39.14918339985888</v>
+        <v>37.8168758994434</v>
       </c>
       <c r="AC285" t="n">
         <v>5391</v>
@@ -33081,13 +33081,13 @@
         <v>10.34391120029613</v>
       </c>
       <c r="Z286" t="n">
-        <v>1.453126400243491</v>
+        <v>0.1234610999235883</v>
       </c>
       <c r="AA286" t="n">
         <v>16.62304340000264</v>
       </c>
       <c r="AB286" t="n">
-        <v>29.59582700044848</v>
+        <v>28.26616170012858</v>
       </c>
       <c r="AC286" t="n">
         <v>4588</v>
@@ -33199,13 +33199,13 @@
         <v>14.52501809969544</v>
       </c>
       <c r="Z287" t="n">
-        <v>3.339925899636</v>
+        <v>0.3506596994120628</v>
       </c>
       <c r="AA287" t="n">
         <v>9.099793700035661</v>
       </c>
       <c r="AB287" t="n">
-        <v>28.49541769933421</v>
+        <v>25.50615149911027</v>
       </c>
       <c r="AC287" t="n">
         <v>2060</v>
@@ -33317,13 +33317,13 @@
         <v>13.95976330013946</v>
       </c>
       <c r="Z288" t="n">
-        <v>1.278361500240862</v>
+        <v>0.05573970021214336</v>
       </c>
       <c r="AA288" t="n">
         <v>7.744470600038767</v>
       </c>
       <c r="AB288" t="n">
-        <v>24.25413600041065</v>
+        <v>23.03151420038193</v>
       </c>
       <c r="AC288" t="n">
         <v>2062</v>
@@ -33435,13 +33435,13 @@
         <v>11.64919309969991</v>
       </c>
       <c r="Z289" t="n">
-        <v>1.697499500121921</v>
+        <v>0.08972390030976385</v>
       </c>
       <c r="AA289" t="n">
         <v>43.3735990000423</v>
       </c>
       <c r="AB289" t="n">
-        <v>57.13051069981884</v>
+        <v>55.52273510000668</v>
       </c>
       <c r="AC289" t="n">
         <v>2061</v>
@@ -33558,13 +33558,13 @@
         <v>14.74588329996914</v>
       </c>
       <c r="Z290" t="n">
-        <v>1.502032100223005</v>
+        <v>0.1142025996232405</v>
       </c>
       <c r="AA290" t="n">
         <v>47.72249849990476</v>
       </c>
       <c r="AB290" t="n">
-        <v>64.71372820029501</v>
+        <v>63.32589869969524</v>
       </c>
       <c r="AC290" t="n">
         <v>2068</v>
@@ -33684,13 +33684,13 @@
         <v>9.92442229995504</v>
       </c>
       <c r="Z291" t="n">
-        <v>2.123013299424201</v>
+        <v>0.1343315999256447</v>
       </c>
       <c r="AA291" t="n">
         <v>44.37449580000248</v>
       </c>
       <c r="AB291" t="n">
-        <v>57.17131599935237</v>
+        <v>55.18263429985382</v>
       </c>
       <c r="AC291" t="n">
         <v>4335</v>
@@ -33806,13 +33806,13 @@
         <v>15.08769860025495</v>
       </c>
       <c r="Z292" t="n">
-        <v>1.917308299802244</v>
+        <v>0.1141757002333179</v>
       </c>
       <c r="AA292" t="n">
         <v>47.16690479998942</v>
       </c>
       <c r="AB292" t="n">
-        <v>65.25195730000269</v>
+        <v>63.44882470043376</v>
       </c>
       <c r="AC292" t="n">
         <v>4986</v>
@@ -33927,13 +33927,13 @@
         <v>10.13664379995316</v>
       </c>
       <c r="Z293" t="n">
-        <v>1.914551499299705</v>
+        <v>0.1575131996069103</v>
       </c>
       <c r="AA293" t="n">
         <v>47.24540769995656</v>
       </c>
       <c r="AB293" t="n">
-        <v>60.32964249921497</v>
+        <v>58.57260419952217</v>
       </c>
       <c r="AC293" t="n">
         <v>2066</v>
@@ -34049,13 +34049,13 @@
         <v>11.25779439974576</v>
       </c>
       <c r="Z294" t="n">
-        <v>1.439926699735224</v>
+        <v>0.1374910994200036</v>
       </c>
       <c r="AA294" t="n">
         <v>42.91062550002243</v>
       </c>
       <c r="AB294" t="n">
-        <v>56.89475459954701</v>
+        <v>55.59231899923179</v>
       </c>
       <c r="AC294" t="n">
         <v>2067</v>
@@ -34176,13 +34176,13 @@
         <v>8.697331599891186</v>
       </c>
       <c r="Z295" t="n">
-        <v>2.248642999213189</v>
+        <v>0.1518364991061389</v>
       </c>
       <c r="AA295" t="n">
         <v>43.6831106999889</v>
       </c>
       <c r="AB295" t="n">
-        <v>57.22185279906262</v>
+        <v>55.12504629895557</v>
       </c>
       <c r="AC295" t="n">
         <v>2068</v>
@@ -34299,13 +34299,13 @@
         <v>10.31776810018346</v>
       </c>
       <c r="Z296" t="n">
-        <v>1.303002000320703</v>
+        <v>0.1327781998552382</v>
       </c>
       <c r="AA296" t="n">
         <v>46.23612240003422</v>
       </c>
       <c r="AB296" t="n">
-        <v>60.60770600044634</v>
+        <v>59.43748219998088</v>
       </c>
       <c r="AC296" t="n">
         <v>2067</v>
@@ -34427,13 +34427,13 @@
         <v>10.22806580038741</v>
       </c>
       <c r="Z297" t="n">
-        <v>1.946034900844097</v>
+        <v>0.2252619009232149</v>
       </c>
       <c r="AA297" t="n">
         <v>46.38257669995073</v>
       </c>
       <c r="AB297" t="n">
-        <v>61.30423120129853</v>
+        <v>59.58345820137765</v>
       </c>
       <c r="AC297" t="n">
         <v>2065</v>
@@ -34545,13 +34545,13 @@
         <v>12.97948159975931</v>
       </c>
       <c r="Z298" t="n">
-        <v>2.616468300111592</v>
+        <v>0.207371799973771</v>
       </c>
       <c r="AA298" t="n">
         <v>43.29790249990765</v>
       </c>
       <c r="AB298" t="n">
-        <v>62.17139979987405</v>
+        <v>59.76230329973623</v>
       </c>
       <c r="AC298" t="n">
         <v>2065</v>
@@ -34663,13 +34663,13 @@
         <v>12.89505390031263</v>
       </c>
       <c r="Z299" t="n">
-        <v>2.231993499677628</v>
+        <v>0.1777909003430977</v>
       </c>
       <c r="AA299" t="n">
         <v>27.04978469992056</v>
       </c>
       <c r="AB299" t="n">
-        <v>45.70095009997021</v>
+        <v>43.64674750063568</v>
       </c>
       <c r="AC299" t="n">
         <v>2066</v>
@@ -34788,13 +34788,13 @@
         <v>10.67095760023221</v>
       </c>
       <c r="Z300" t="n">
-        <v>1.207375900354236</v>
+        <v>0.05532860057428479</v>
       </c>
       <c r="AA300" t="n">
         <v>28.76099149999209</v>
       </c>
       <c r="AB300" t="n">
-        <v>43.9258862005081</v>
+        <v>42.77383890072815</v>
       </c>
       <c r="AC300" t="n">
         <v>2070</v>
@@ -34906,13 +34906,13 @@
         <v>8.217519299592823</v>
       </c>
       <c r="Z301" t="n">
-        <v>1.183793200179935</v>
+        <v>0.1272172001190484</v>
       </c>
       <c r="AA301" t="n">
         <v>26.74349289992824</v>
       </c>
       <c r="AB301" t="n">
-        <v>39.5522680998547</v>
+        <v>38.49569209979381</v>
       </c>
       <c r="AC301" t="n">
         <v>2068</v>
@@ -35068,10 +35068,10 @@
         <v>676.77251870092</v>
       </c>
       <c r="C10" t="n">
-        <v>866.7278056973591</v>
+        <v>821.4861965975724</v>
       </c>
       <c r="D10" t="n">
-        <v>4724.015682603465</v>
+        <v>4458.696156195947</v>
       </c>
     </row>
     <row r="11">
@@ -35449,10 +35449,10 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.4786859189951793</v>
+        <v>0.02626982799731195</v>
       </c>
       <c r="D35" t="n">
-        <v>2.866435058019124</v>
+        <v>0.2132397939439397</v>
       </c>
     </row>
     <row r="36">
@@ -35481,10 +35481,10 @@
         <v>6.767725187009201</v>
       </c>
       <c r="C37" t="n">
-        <v>8.667278056973592</v>
+        <v>8.214861965975723</v>
       </c>
       <c r="D37" t="n">
-        <v>47.24015682603466</v>
+        <v>44.58696156195947</v>
       </c>
     </row>
     <row r="38">
@@ -36151,7 +36151,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RAGAS NonLLMContextRecall. Relevant contexts retrieved / all reference contexts. Relevant: Levenshtein similarity to a reference context of 0.5 or more. Reference context: text of a HERB evidence record.</t>
+          <t>RAGAS NonLLMContextRecall. Relevant contexts retrieved / all reference contexts. Relevant: Levenshtein similarity to a reference context of more than 0.5. Reference context: the content of a HERB evidence record, without ids, labels, dates and names. Retrieved contexts: the content of each record passed to the answer model.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -36173,7 +36173,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>RAGAS NonLLMContextPrecisionWithReference. Context precision@K: mean of precision@k over the ranks k of the relevant retrieved contexts. Relevant: Levenshtein similarity to a reference context of 0.5 or more.</t>
+          <t>RAGAS NonLLMContextPrecisionWithReference. Context precision@K: mean of precision@k over the ranks k of the relevant retrieved contexts. Relevant: Levenshtein similarity to a reference context of 0.5 or more. Reference context: the content of a HERB evidence record, without ids, labels, dates and names. Retrieved contexts: the content of each record passed to the answer model.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">

</xml_diff>